<commit_message>
Ajout du reste libre, des charges perso (détail ou forfait) et de l'épargne perso
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KqkJNWVZSWN9upSPoUaH5h
</commit_message>
<xml_diff>
--- a/suivi_comptes.xlsx
+++ b/suivi_comptes.xlsx
@@ -13,6 +13,7 @@
     <sheet name="Comptes" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Charges" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Revenus" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Charges perso" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="139">
   <si>
     <t xml:space="preserve">Synthèse mensuelle</t>
   </si>
@@ -53,7 +54,19 @@
     <t xml:space="preserve">Taux d'effort</t>
   </si>
   <si>
-    <t xml:space="preserve">Reste à vivre (solde du compte perso)</t>
+    <t xml:space="preserve">Reste après charges communes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Charges perso (détail ou forfait)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reste après charges perso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Épargne perso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reste libre (loisirs…)</t>
   </si>
   <si>
     <t xml:space="preserve">Total foyer</t>
@@ -95,6 +108,15 @@
     <t xml:space="preserve">Lecture : un compte joint à solde 0 est équilibré. Un compte perso à solde positif = reste à vivre ; négatif = salaire insuffisant. Les aides sont réparties sur les deux personnes au prorata de leurs parts de charges (hypothèse).</t>
   </si>
   <si>
+    <t xml:space="preserve">3. Charges communes : fixe vs variable (mensuel)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fixe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Variable / estimé</t>
+  </si>
+  <si>
     <t xml:space="preserve">Paramètres du foyer</t>
   </si>
   <si>
@@ -152,6 +174,39 @@
     <t xml:space="preserve">Modes de répartition possibles : 50/50 · Prorata salaires · Personne 1 seul · Personne 2 seul</t>
   </si>
   <si>
+    <t xml:space="preserve">Budget personnel (le « reste libre »)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Charges perso : mode (Détail = onglet « Charges perso » ; Forfait = somme arbitraire)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Détail</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forfait</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forfait charges perso (€/mois), utilisé si mode Forfait</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Épargne perso : mode (Pourcentage ou Montant)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pourcentage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Montant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Épargne perso : pourcentage du reste (si Pourcentage)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Épargne perso : montant €/mois (si Montant)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Si l'un de vous ne veut pas détailler ses comptes : mode Forfait + une somme. Ses lignes éventuelles dans « Charges perso » sont alors ignorées.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Comptes bancaires</t>
   </si>
   <si>
@@ -212,7 +267,7 @@
     <t xml:space="preserve">Charges (dépenses récurrentes)</t>
   </si>
   <si>
-    <t xml:space="preserve">Remplir les colonnes jaunes (50 lignes). Montant = montant par période ; le mensuel et les parts se calculent. Virement : indiquer le compte destinataire (liste libre).</t>
+    <t xml:space="preserve">Remplir les colonnes jaunes (50 lignes). Montant = montant par période ; le mensuel et les parts se calculent. Virement : indiquer le compte destinataire (liste libre). Dépenses irrégulières : saisir une enveloppe annuelle, elle est lissée par mois.</t>
   </si>
   <si>
     <t xml:space="preserve">Libellé</t>
@@ -254,9 +309,6 @@
     <t xml:space="preserve">Logement</t>
   </si>
   <si>
-    <t xml:space="preserve">Fixe</t>
-  </si>
-  <si>
     <t xml:space="preserve">Prélèvement</t>
   </si>
   <si>
@@ -326,6 +378,21 @@
     <t xml:space="preserve">Mairie (cantine)</t>
   </si>
   <si>
+    <t xml:space="preserve">Vêtements enfants (enveloppe lissée)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Médecin / pharmacie (provision)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Santé</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cadeaux &amp; fêtes (enveloppe lissée)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loisirs</t>
+  </si>
+  <si>
     <t xml:space="preserve">TOTAL mensuel</t>
   </si>
   <si>
@@ -357,6 +424,24 @@
   </si>
   <si>
     <t xml:space="preserve">Prime d'activité (CAF)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Charges personnelles (facultatif)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dépenses propres à chacun. Utilisé seulement si le mode « Détail » est choisi pour la personne dans Paramètres.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Salle de sport</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coiffeur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Soins</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abonnement musique</t>
   </si>
 </sst>
 </file>
@@ -369,7 +454,7 @@
     <numFmt numFmtId="166" formatCode="0%"/>
     <numFmt numFmtId="167" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -449,6 +534,12 @@
     <font>
       <sz val="10"/>
       <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -536,7 +627,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="21">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -601,11 +692,23 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="165" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -861,7 +964,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:K30"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
@@ -871,7 +974,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="10" style="0" width="18"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -911,6 +1014,18 @@
       <c r="G4" s="4" t="s">
         <v>9</v>
       </c>
+      <c r="H4" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="str">
@@ -923,7 +1038,7 @@
       </c>
       <c r="C5" s="6" t="n">
         <f aca="false">SUM(E$13:E$22)</f>
-        <v>1170.9794275492</v>
+        <v>1232.85600681269</v>
       </c>
       <c r="D5" s="6" t="n">
         <f aca="false">IFERROR(INDEX($C$13:$C$22,MATCH(Paramètres!$B$6,$A$13:$A$22,0)),0)</f>
@@ -931,15 +1046,31 @@
       </c>
       <c r="E5" s="6" t="n">
         <f aca="false">C5+D5</f>
-        <v>1170.9794275492</v>
+        <v>1232.85600681269</v>
       </c>
       <c r="F5" s="7" t="n">
         <f aca="false">IF(B5=0,0,E5/B5)</f>
-        <v>0.487908094812165</v>
+        <v>0.51369000283862</v>
       </c>
       <c r="G5" s="6" t="n">
         <f aca="false">IFERROR(INDEX($J$13:$J$22,MATCH(Paramètres!$B$6,$A$13:$A$22,0)),0)</f>
-        <v>1229.02057245081</v>
+        <v>1167.14399318731</v>
+      </c>
+      <c r="H5" s="6" t="n">
+        <f aca="false">IF(Paramètres!B$15="Forfait",Paramètres!B$16,SUMIFS('Charges perso'!$F$5:$F$44,'Charges perso'!$B$5:$B$44,A5))</f>
+        <v>86</v>
+      </c>
+      <c r="I5" s="6" t="n">
+        <f aca="false">G5-H5</f>
+        <v>1081.14399318731</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <f aca="false">MAX(0,IF(Paramètres!B$17="Pourcentage",Paramètres!B$18*MAX(0,I5),Paramètres!B$19))</f>
+        <v>324.343197956193</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <f aca="false">I5-J5</f>
+        <v>756.800795231118</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -953,7 +1084,7 @@
       </c>
       <c r="C6" s="6" t="n">
         <f aca="false">SUM(F$13:F$22)</f>
-        <v>972.353905784138</v>
+        <v>1032.14399318731</v>
       </c>
       <c r="D6" s="6" t="n">
         <f aca="false">IFERROR(INDEX($C$13:$C$22,MATCH(Paramètres!$B$7,$A$13:$A$22,0)),0)</f>
@@ -961,20 +1092,36 @@
       </c>
       <c r="E6" s="6" t="n">
         <f aca="false">C6+D6</f>
-        <v>1000.35390578414</v>
+        <v>1060.14399318731</v>
       </c>
       <c r="F6" s="7" t="n">
         <f aca="false">IF(B6=0,0,E6/B6)</f>
-        <v>0.526502055675862</v>
+        <v>0.557970522730164</v>
       </c>
       <c r="G6" s="6" t="n">
         <f aca="false">IFERROR(INDEX($J$13:$J$22,MATCH(Paramètres!$B$7,$A$13:$A$22,0)),0)</f>
-        <v>899.646094215862</v>
+        <v>839.856006812689</v>
+      </c>
+      <c r="H6" s="6" t="n">
+        <f aca="false">IF(Paramètres!C$15="Forfait",Paramètres!C$16,SUMIFS('Charges perso'!$F$5:$F$44,'Charges perso'!$B$5:$B$44,A6))</f>
+        <v>350</v>
+      </c>
+      <c r="I6" s="6" t="n">
+        <f aca="false">G6-H6</f>
+        <v>489.856006812689</v>
+      </c>
+      <c r="J6" s="6" t="n">
+        <f aca="false">MAX(0,IF(Paramètres!C$17="Pourcentage",Paramètres!C$18*MAX(0,I6),Paramètres!C$19))</f>
+        <v>200</v>
+      </c>
+      <c r="K6" s="6" t="n">
+        <f aca="false">I6-J6</f>
+        <v>289.856006812689</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B7" s="9" t="n">
         <f aca="false">SUM(B5:B6)</f>
@@ -982,7 +1129,7 @@
       </c>
       <c r="C7" s="9" t="n">
         <f aca="false">SUM(C5:C6)</f>
-        <v>2143.33333333333</v>
+        <v>2265</v>
       </c>
       <c r="D7" s="9" t="n">
         <f aca="false">SUM(D5:D6)</f>
@@ -990,39 +1137,55 @@
       </c>
       <c r="E7" s="9" t="n">
         <f aca="false">SUM(E5:E6)</f>
-        <v>2171.33333333333</v>
+        <v>2293</v>
       </c>
       <c r="F7" s="10" t="n">
         <f aca="false">IF(B7=0,0,E7/B7)</f>
-        <v>0.504961240310078</v>
+        <v>0.533255813953488</v>
       </c>
       <c r="G7" s="9" t="n">
         <f aca="false">SUM(G5:G6)</f>
-        <v>2128.66666666667</v>
+        <v>2007</v>
+      </c>
+      <c r="H7" s="9" t="n">
+        <f aca="false">SUM(H5:H6)</f>
+        <v>436</v>
+      </c>
+      <c r="I7" s="9" t="n">
+        <f aca="false">SUM(I5:I6)</f>
+        <v>1571</v>
+      </c>
+      <c r="J7" s="9" t="n">
+        <f aca="false">SUM(J5:J6)</f>
+        <v>524.343197956193</v>
+      </c>
+      <c r="K7" s="9" t="n">
+        <f aca="false">SUM(K5:K6)</f>
+        <v>1046.65680204381</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E12" s="4" t="str">
         <f aca="false">"À virer par "&amp;Paramètres!$B$4</f>
@@ -1033,16 +1196,16 @@
         <v>À virer par Sam</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="I12" s="4" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="J12" s="4" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1080,11 +1243,11 @@
       </c>
       <c r="I13" s="6" t="n">
         <f aca="false">IF($A13="","",IF($A13=Paramètres!$B$6,SUM($E$13:$E$22),IF($A13=Paramètres!$B$7,SUM($F$13:$F$22),0)))</f>
-        <v>1170.9794275492</v>
+        <v>1232.85600681269</v>
       </c>
       <c r="J13" s="6" t="n">
         <f aca="false">IF($A13="","",G13+D13+H13+IF(B13="Joint",E13+F13,0)-C13-I13)</f>
-        <v>1229.02057245081</v>
+        <v>1167.14399318731</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1122,11 +1285,11 @@
       </c>
       <c r="I14" s="6" t="n">
         <f aca="false">IF($A14="","",IF($A14=Paramètres!$B$6,SUM($E$13:$E$22),IF($A14=Paramètres!$B$7,SUM($F$13:$F$22),0)))</f>
-        <v>972.353905784138</v>
+        <v>1032.14399318731</v>
       </c>
       <c r="J14" s="6" t="n">
         <f aca="false">IF($A14="","",G14+D14+H14+IF(B14="Joint",E14+F14,0)-C14-I14)</f>
-        <v>899.646094215862</v>
+        <v>839.856006812689</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1182,7 +1345,7 @@
       </c>
       <c r="C16" s="6" t="n">
         <f aca="false">IF($A16="","",SUMIFS(Charges!$F$5:$F$54,Charges!$H$5:$H$54,$A16))</f>
-        <v>910</v>
+        <v>1031.66666666667</v>
       </c>
       <c r="D16" s="6" t="n">
         <f aca="false">IF($A16="","",SUMIFS(Revenus!$F$5:$F$24,Revenus!$G$5:$G$24,$A16,Revenus!$B$5:$B$24,"&lt;&gt;Salaire"))</f>
@@ -1190,11 +1353,11 @@
       </c>
       <c r="E16" s="11" t="n">
         <f aca="false">IF($A16="","",IF($B16="Joint",IF($C16=0,0,($C16-$D16)*SUMIFS(Charges!$M$5:$M$54,Charges!$H$5:$H$54,$A16)/$C16),0))</f>
-        <v>366.153846153846</v>
+        <v>428.03042541734</v>
       </c>
       <c r="F16" s="11" t="n">
         <f aca="false">IF($A16="","",IF($B16="Joint",IF($C16=0,0,($C16-$D16)*SUMIFS(Charges!$N$5:$N$54,Charges!$H$5:$H$54,$A16)/$C16),0))</f>
-        <v>313.846153846154</v>
+        <v>373.636241249327</v>
       </c>
       <c r="G16" s="6" t="n">
         <f aca="false">IF($A16="","",SUMIFS(Revenus!$F$5:$F$24,Revenus!$G$5:$G$24,$A16,Revenus!$B$5:$B$24,"Salaire"))</f>
@@ -1467,12 +1630,12 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="8" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B23" s="8"/>
       <c r="C23" s="9" t="n">
         <f aca="false">SUM(C13:C22)</f>
-        <v>2401.33333333333</v>
+        <v>2523</v>
       </c>
       <c r="D23" s="9" t="n">
         <f aca="false">SUM(D13:D22)</f>
@@ -1480,11 +1643,11 @@
       </c>
       <c r="E23" s="9" t="n">
         <f aca="false">SUM(E13:E22)</f>
-        <v>1170.9794275492</v>
+        <v>1232.85600681269</v>
       </c>
       <c r="F23" s="9" t="n">
         <f aca="false">SUM(F13:F22)</f>
-        <v>972.353905784138</v>
+        <v>1032.14399318731</v>
       </c>
       <c r="G23" s="9" t="n">
         <f aca="false">SUM(G13:G22)</f>
@@ -1496,16 +1659,60 @@
       </c>
       <c r="I23" s="9" t="n">
         <f aca="false">SUM(I13:I22)</f>
-        <v>2143.33333333333</v>
+        <v>2265</v>
       </c>
       <c r="J23" s="9" t="n">
         <f aca="false">SUM(J13:J22)</f>
-        <v>2278.66666666667</v>
+        <v>2157</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>22</v>
+        <v>26</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B28" s="6" t="n">
+        <f aca="false">SUMIFS(Charges!$F$5:$F$54,Charges!$C$5:$C$54,"Fixe")</f>
+        <v>1581.33333333333</v>
+      </c>
+      <c r="C28" s="7" t="n">
+        <f aca="false">IF($B$30=0,0,B28/$B$30)</f>
+        <v>0.626767076231999</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B29" s="6" t="n">
+        <f aca="false">SUMIFS(Charges!$F$5:$F$54,Charges!$C$5:$C$54,"Variable")</f>
+        <v>941.666666666667</v>
+      </c>
+      <c r="C29" s="7" t="n">
+        <f aca="false">IF($B$30=0,0,B29/$B$30)</f>
+        <v>0.373232923768001</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="B30" s="9" t="n">
+        <f aca="false">B28+B29</f>
+        <v>2523</v>
+      </c>
+      <c r="C30" s="10" t="n">
+        <f aca="false">C28+C29</f>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1524,43 +1731,42 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>24</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D3" s="12" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="E3" s="12" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="E4" s="5" t="n">
         <v>1</v>
@@ -1568,13 +1774,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="12" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="E5" s="5" t="n">
         <v>3</v>
@@ -1582,13 +1788,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="E6" s="5" t="n">
         <v>6</v>
@@ -1596,13 +1802,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="E7" s="5" t="n">
         <v>12</v>
@@ -1610,7 +1816,7 @@
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="B9" s="15" t="n">
         <f aca="false">IFERROR(SUMIFS(Revenus!$F$5:$F$24,Revenus!$B$5:$B$24,"Salaire",Revenus!$C$5:$C$24,$B$4)/SUMIFS(Revenus!$F$5:$F$24,Revenus!$B$5:$B$24,"Salaire"),0.5)</f>
@@ -1619,15 +1825,98 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>41</v>
+        <v>48</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B14" s="16" t="str">
+        <f aca="false">$B$4</f>
+        <v>Alex</v>
+      </c>
+      <c r="C14" s="16" t="str">
+        <f aca="false">$B$5</f>
+        <v>Sam</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="17" t="s">
+        <v>50</v>
+      </c>
+      <c r="B15" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="C15" s="13" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="17" t="s">
+        <v>53</v>
+      </c>
+      <c r="B16" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="18" t="n">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="B17" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="C17" s="13" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="B18" s="19" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C18" s="19" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="17" t="s">
+        <v>58</v>
+      </c>
+      <c r="B19" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="18" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="2" t="s">
+        <v>59</v>
       </c>
     </row>
   </sheetData>
+  <dataValidations count="2">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B15:C15" type="list">
+      <formula1>"Détail,Forfait"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B17:C17" type="list">
+      <formula1>"Pourcentage,Montant"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -1654,110 +1943,110 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>42</v>
+        <v>60</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>43</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>44</v>
+        <v>62</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>45</v>
+        <v>63</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>46</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>47</v>
+        <v>65</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>48</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>47</v>
+        <v>65</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>50</v>
+        <v>68</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>51</v>
+        <v>69</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>53</v>
+        <v>71</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>54</v>
+        <v>72</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>51</v>
+        <v>69</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>55</v>
+        <v>73</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>51</v>
+        <v>69</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>59</v>
+        <v>77</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>60</v>
+        <v>78</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1825,50 +2114,50 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>62</v>
+        <v>80</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>63</v>
+        <v>81</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>64</v>
+        <v>82</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>65</v>
+        <v>83</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>67</v>
+        <v>85</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>68</v>
+        <v>86</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>69</v>
+        <v>87</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>70</v>
+        <v>88</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>71</v>
+        <v>89</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>72</v>
+        <v>90</v>
       </c>
       <c r="L4" s="4" t="s">
-        <v>73</v>
+        <v>91</v>
       </c>
       <c r="M4" s="4" t="str">
         <f aca="false">"Part "&amp;Paramètres!$B$4&amp;" (€/mois)"</f>
@@ -1881,18 +2170,18 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>74</v>
+        <v>92</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>75</v>
+        <v>93</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>76</v>
+        <v>28</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="E5" s="16" t="n">
+        <v>36</v>
+      </c>
+      <c r="E5" s="18" t="n">
         <v>1150</v>
       </c>
       <c r="F5" s="6" t="n">
@@ -1900,17 +2189,17 @@
         <v>1150</v>
       </c>
       <c r="G5" s="13" t="s">
-        <v>77</v>
+        <v>94</v>
       </c>
       <c r="H5" s="13" t="s">
-        <v>50</v>
+        <v>68</v>
       </c>
       <c r="I5" s="13"/>
       <c r="J5" s="13" t="n">
         <v>5</v>
       </c>
       <c r="K5" s="13" t="s">
-        <v>78</v>
+        <v>95</v>
       </c>
       <c r="L5" s="7" t="n">
         <f aca="false">IF(A5="","",IF(K5="50/50",0.5,IF(K5="Prorata salaires",Paramètres!$B$9,IF(K5="Personne 1 seul",1,IF(K5="Personne 2 seul",0,0.5)))))</f>
@@ -1927,18 +2216,18 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>75</v>
+        <v>93</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>76</v>
+        <v>28</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="E6" s="16" t="n">
+        <v>36</v>
+      </c>
+      <c r="E6" s="18" t="n">
         <v>45</v>
       </c>
       <c r="F6" s="6" t="n">
@@ -1946,17 +2235,17 @@
         <v>45</v>
       </c>
       <c r="G6" s="13" t="s">
-        <v>77</v>
+        <v>94</v>
       </c>
       <c r="H6" s="13" t="s">
-        <v>50</v>
+        <v>68</v>
       </c>
       <c r="I6" s="13"/>
       <c r="J6" s="13" t="n">
         <v>5</v>
       </c>
       <c r="K6" s="13" t="s">
-        <v>80</v>
+        <v>97</v>
       </c>
       <c r="L6" s="7" t="n">
         <f aca="false">IF(A6="","",IF(K6="50/50",0.5,IF(K6="Prorata salaires",Paramètres!$B$9,IF(K6="Personne 1 seul",1,IF(K6="Personne 2 seul",0,0.5)))))</f>
@@ -1973,18 +2262,18 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>81</v>
+        <v>98</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>75</v>
+        <v>93</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>76</v>
+        <v>28</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>38</v>
-      </c>
-      <c r="E7" s="16" t="n">
+        <v>45</v>
+      </c>
+      <c r="E7" s="18" t="n">
         <v>1300</v>
       </c>
       <c r="F7" s="6" t="n">
@@ -1992,17 +2281,17 @@
         <v>108.333333333333</v>
       </c>
       <c r="G7" s="13" t="s">
-        <v>77</v>
+        <v>94</v>
       </c>
       <c r="H7" s="13" t="s">
-        <v>50</v>
+        <v>68</v>
       </c>
       <c r="I7" s="13"/>
       <c r="J7" s="13" t="n">
         <v>15</v>
       </c>
       <c r="K7" s="13" t="s">
-        <v>78</v>
+        <v>95</v>
       </c>
       <c r="L7" s="7" t="n">
         <f aca="false">IF(A7="","",IF(K7="50/50",0.5,IF(K7="Prorata salaires",Paramètres!$B$9,IF(K7="Personne 1 seul",1,IF(K7="Personne 2 seul",0,0.5)))))</f>
@@ -2019,18 +2308,18 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>82</v>
+        <v>99</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>83</v>
+        <v>100</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="E8" s="16" t="n">
+        <v>36</v>
+      </c>
+      <c r="E8" s="18" t="n">
         <v>130</v>
       </c>
       <c r="F8" s="6" t="n">
@@ -2038,17 +2327,17 @@
         <v>130</v>
       </c>
       <c r="G8" s="13" t="s">
-        <v>77</v>
+        <v>94</v>
       </c>
       <c r="H8" s="13" t="s">
-        <v>50</v>
+        <v>68</v>
       </c>
       <c r="I8" s="13"/>
       <c r="J8" s="13" t="n">
         <v>12</v>
       </c>
       <c r="K8" s="13" t="s">
-        <v>80</v>
+        <v>97</v>
       </c>
       <c r="L8" s="7" t="n">
         <f aca="false">IF(A8="","",IF(K8="50/50",0.5,IF(K8="Prorata salaires",Paramètres!$B$9,IF(K8="Personne 1 seul",1,IF(K8="Personne 2 seul",0,0.5)))))</f>
@@ -2065,18 +2354,18 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>85</v>
+        <v>102</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>86</v>
+        <v>103</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>76</v>
+        <v>28</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="E9" s="16" t="n">
+        <v>36</v>
+      </c>
+      <c r="E9" s="18" t="n">
         <v>30</v>
       </c>
       <c r="F9" s="6" t="n">
@@ -2084,17 +2373,17 @@
         <v>30</v>
       </c>
       <c r="G9" s="13" t="s">
-        <v>77</v>
+        <v>94</v>
       </c>
       <c r="H9" s="13" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="I9" s="13"/>
       <c r="J9" s="13" t="n">
         <v>10</v>
       </c>
       <c r="K9" s="13" t="s">
-        <v>80</v>
+        <v>97</v>
       </c>
       <c r="L9" s="7" t="n">
         <f aca="false">IF(A9="","",IF(K9="50/50",0.5,IF(K9="Prorata salaires",Paramètres!$B$9,IF(K9="Personne 1 seul",1,IF(K9="Personne 2 seul",0,0.5)))))</f>
@@ -2111,18 +2400,18 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>76</v>
+        <v>28</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>32</v>
-      </c>
-      <c r="E10" s="16" t="n">
+        <v>39</v>
+      </c>
+      <c r="E10" s="18" t="n">
         <v>210</v>
       </c>
       <c r="F10" s="6" t="n">
@@ -2130,17 +2419,17 @@
         <v>70</v>
       </c>
       <c r="G10" s="13" t="s">
-        <v>77</v>
+        <v>94</v>
       </c>
       <c r="H10" s="13" t="s">
-        <v>54</v>
+        <v>72</v>
       </c>
       <c r="I10" s="13"/>
       <c r="J10" s="13" t="n">
         <v>1</v>
       </c>
       <c r="K10" s="13" t="s">
-        <v>89</v>
+        <v>106</v>
       </c>
       <c r="L10" s="7" t="n">
         <f aca="false">IF(A10="","",IF(K10="50/50",0.5,IF(K10="Prorata salaires",Paramètres!$B$9,IF(K10="Personne 1 seul",1,IF(K10="Personne 2 seul",0,0.5)))))</f>
@@ -2157,18 +2446,18 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>90</v>
+        <v>107</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>86</v>
+        <v>103</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>76</v>
+        <v>28</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="E11" s="16" t="n">
+        <v>36</v>
+      </c>
+      <c r="E11" s="18" t="n">
         <v>28</v>
       </c>
       <c r="F11" s="6" t="n">
@@ -2176,17 +2465,17 @@
         <v>28</v>
       </c>
       <c r="G11" s="13" t="s">
-        <v>77</v>
+        <v>94</v>
       </c>
       <c r="H11" s="13" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="I11" s="13"/>
       <c r="J11" s="13" t="n">
         <v>8</v>
       </c>
       <c r="K11" s="13" t="s">
-        <v>91</v>
+        <v>108</v>
       </c>
       <c r="L11" s="7" t="n">
         <f aca="false">IF(A11="","",IF(K11="50/50",0.5,IF(K11="Prorata salaires",Paramètres!$B$9,IF(K11="Personne 1 seul",1,IF(K11="Personne 2 seul",0,0.5)))))</f>
@@ -2203,18 +2492,18 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>92</v>
+        <v>109</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>93</v>
+        <v>110</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="E12" s="16" t="n">
+        <v>36</v>
+      </c>
+      <c r="E12" s="18" t="n">
         <v>600</v>
       </c>
       <c r="F12" s="6" t="n">
@@ -2222,15 +2511,15 @@
         <v>600</v>
       </c>
       <c r="G12" s="13" t="s">
-        <v>94</v>
+        <v>111</v>
       </c>
       <c r="H12" s="13" t="s">
-        <v>54</v>
+        <v>72</v>
       </c>
       <c r="I12" s="13"/>
       <c r="J12" s="13"/>
       <c r="K12" s="13" t="s">
-        <v>80</v>
+        <v>97</v>
       </c>
       <c r="L12" s="7" t="n">
         <f aca="false">IF(A12="","",IF(K12="50/50",0.5,IF(K12="Prorata salaires",Paramètres!$B$9,IF(K12="Personne 1 seul",1,IF(K12="Personne 2 seul",0,0.5)))))</f>
@@ -2247,18 +2536,18 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>95</v>
+        <v>112</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>59</v>
+        <v>77</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>76</v>
+        <v>28</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="E13" s="16" t="n">
+        <v>36</v>
+      </c>
+      <c r="E13" s="18" t="n">
         <v>150</v>
       </c>
       <c r="F13" s="6" t="n">
@@ -2266,19 +2555,19 @@
         <v>150</v>
       </c>
       <c r="G13" s="13" t="s">
-        <v>96</v>
+        <v>113</v>
       </c>
       <c r="H13" s="13" t="s">
-        <v>54</v>
+        <v>72</v>
       </c>
       <c r="I13" s="13" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="J13" s="13" t="n">
         <v>3</v>
       </c>
       <c r="K13" s="13" t="s">
-        <v>80</v>
+        <v>97</v>
       </c>
       <c r="L13" s="7" t="n">
         <f aca="false">IF(A13="","",IF(K13="50/50",0.5,IF(K13="Prorata salaires",Paramètres!$B$9,IF(K13="Personne 1 seul",1,IF(K13="Personne 2 seul",0,0.5)))))</f>
@@ -2295,18 +2584,18 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>97</v>
+        <v>114</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>98</v>
+        <v>115</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="E14" s="16" t="n">
+        <v>36</v>
+      </c>
+      <c r="E14" s="18" t="n">
         <v>90</v>
       </c>
       <c r="F14" s="6" t="n">
@@ -2314,19 +2603,19 @@
         <v>90</v>
       </c>
       <c r="G14" s="13" t="s">
-        <v>96</v>
+        <v>113</v>
       </c>
       <c r="H14" s="13" t="s">
-        <v>54</v>
+        <v>72</v>
       </c>
       <c r="I14" s="13" t="s">
-        <v>99</v>
+        <v>116</v>
       </c>
       <c r="J14" s="13" t="n">
         <v>28</v>
       </c>
       <c r="K14" s="13" t="s">
-        <v>80</v>
+        <v>97</v>
       </c>
       <c r="L14" s="7" t="n">
         <f aca="false">IF(A14="","",IF(K14="50/50",0.5,IF(K14="Prorata salaires",Paramètres!$B$9,IF(K14="Personne 1 seul",1,IF(K14="Personne 2 seul",0,0.5)))))</f>
@@ -2342,87 +2631,135 @@
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="13"/>
-      <c r="B15" s="13"/>
-      <c r="C15" s="13"/>
-      <c r="D15" s="13"/>
-      <c r="E15" s="16"/>
-      <c r="F15" s="6" t="str">
+      <c r="A15" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="B15" s="13" t="s">
+        <v>115</v>
+      </c>
+      <c r="C15" s="13" t="s">
+        <v>101</v>
+      </c>
+      <c r="D15" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="E15" s="18" t="n">
+        <v>600</v>
+      </c>
+      <c r="F15" s="6" t="n">
         <f aca="false">IF(A15="","",IFERROR(E15/INDEX(Paramètres!$E$4:$E$7,MATCH(D15,Paramètres!$D$4:$D$7,0)),0))</f>
-        <v/>
-      </c>
-      <c r="G15" s="13"/>
-      <c r="H15" s="13"/>
+        <v>50</v>
+      </c>
+      <c r="G15" s="13" t="s">
+        <v>111</v>
+      </c>
+      <c r="H15" s="13" t="s">
+        <v>72</v>
+      </c>
       <c r="I15" s="13"/>
       <c r="J15" s="13"/>
-      <c r="K15" s="13"/>
-      <c r="L15" s="7" t="str">
+      <c r="K15" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="L15" s="7" t="n">
         <f aca="false">IF(A15="","",IF(K15="50/50",0.5,IF(K15="Prorata salaires",Paramètres!$B$9,IF(K15="Personne 1 seul",1,IF(K15="Personne 2 seul",0,0.5)))))</f>
-        <v/>
-      </c>
-      <c r="M15" s="6" t="str">
+        <v>0.5</v>
+      </c>
+      <c r="M15" s="6" t="n">
         <f aca="false">IF(A15="","",F15*L15)</f>
-        <v/>
-      </c>
-      <c r="N15" s="6" t="str">
+        <v>25</v>
+      </c>
+      <c r="N15" s="6" t="n">
         <f aca="false">IF(A15="","",F15-M15)</f>
-        <v/>
+        <v>25</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="13"/>
-      <c r="B16" s="13"/>
-      <c r="C16" s="13"/>
-      <c r="D16" s="13"/>
-      <c r="E16" s="16"/>
-      <c r="F16" s="6" t="str">
+      <c r="A16" s="13" t="s">
+        <v>118</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>101</v>
+      </c>
+      <c r="D16" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="E16" s="18" t="n">
+        <v>30</v>
+      </c>
+      <c r="F16" s="6" t="n">
         <f aca="false">IF(A16="","",IFERROR(E16/INDEX(Paramètres!$E$4:$E$7,MATCH(D16,Paramètres!$D$4:$D$7,0)),0))</f>
-        <v/>
-      </c>
-      <c r="G16" s="13"/>
-      <c r="H16" s="13"/>
+        <v>30</v>
+      </c>
+      <c r="G16" s="13" t="s">
+        <v>111</v>
+      </c>
+      <c r="H16" s="13" t="s">
+        <v>72</v>
+      </c>
       <c r="I16" s="13"/>
       <c r="J16" s="13"/>
-      <c r="K16" s="13"/>
-      <c r="L16" s="7" t="str">
+      <c r="K16" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="L16" s="7" t="n">
         <f aca="false">IF(A16="","",IF(K16="50/50",0.5,IF(K16="Prorata salaires",Paramètres!$B$9,IF(K16="Personne 1 seul",1,IF(K16="Personne 2 seul",0,0.5)))))</f>
-        <v/>
-      </c>
-      <c r="M16" s="6" t="str">
+        <v>0.5</v>
+      </c>
+      <c r="M16" s="6" t="n">
         <f aca="false">IF(A16="","",F16*L16)</f>
-        <v/>
-      </c>
-      <c r="N16" s="6" t="str">
+        <v>15</v>
+      </c>
+      <c r="N16" s="6" t="n">
         <f aca="false">IF(A16="","",F16-M16)</f>
-        <v/>
+        <v>15</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="13"/>
-      <c r="B17" s="13"/>
-      <c r="C17" s="13"/>
-      <c r="D17" s="13"/>
-      <c r="E17" s="16"/>
-      <c r="F17" s="6" t="str">
+      <c r="A17" s="13" t="s">
+        <v>120</v>
+      </c>
+      <c r="B17" s="13" t="s">
+        <v>121</v>
+      </c>
+      <c r="C17" s="13" t="s">
+        <v>101</v>
+      </c>
+      <c r="D17" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="E17" s="18" t="n">
+        <v>500</v>
+      </c>
+      <c r="F17" s="6" t="n">
         <f aca="false">IF(A17="","",IFERROR(E17/INDEX(Paramètres!$E$4:$E$7,MATCH(D17,Paramètres!$D$4:$D$7,0)),0))</f>
-        <v/>
-      </c>
-      <c r="G17" s="13"/>
-      <c r="H17" s="13"/>
+        <v>41.6666666666667</v>
+      </c>
+      <c r="G17" s="13" t="s">
+        <v>111</v>
+      </c>
+      <c r="H17" s="13" t="s">
+        <v>72</v>
+      </c>
       <c r="I17" s="13"/>
       <c r="J17" s="13"/>
-      <c r="K17" s="13"/>
-      <c r="L17" s="7" t="str">
+      <c r="K17" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="L17" s="7" t="n">
         <f aca="false">IF(A17="","",IF(K17="50/50",0.5,IF(K17="Prorata salaires",Paramètres!$B$9,IF(K17="Personne 1 seul",1,IF(K17="Personne 2 seul",0,0.5)))))</f>
-        <v/>
-      </c>
-      <c r="M17" s="6" t="str">
+        <v>0.5</v>
+      </c>
+      <c r="M17" s="6" t="n">
         <f aca="false">IF(A17="","",F17*L17)</f>
-        <v/>
-      </c>
-      <c r="N17" s="6" t="str">
+        <v>20.8333333333333</v>
+      </c>
+      <c r="N17" s="6" t="n">
         <f aca="false">IF(A17="","",F17-M17)</f>
-        <v/>
+        <v>20.8333333333333</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2430,7 +2767,7 @@
       <c r="B18" s="13"/>
       <c r="C18" s="13"/>
       <c r="D18" s="13"/>
-      <c r="E18" s="16"/>
+      <c r="E18" s="18"/>
       <c r="F18" s="6" t="str">
         <f aca="false">IF(A18="","",IFERROR(E18/INDEX(Paramètres!$E$4:$E$7,MATCH(D18,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
@@ -2458,7 +2795,7 @@
       <c r="B19" s="13"/>
       <c r="C19" s="13"/>
       <c r="D19" s="13"/>
-      <c r="E19" s="16"/>
+      <c r="E19" s="18"/>
       <c r="F19" s="6" t="str">
         <f aca="false">IF(A19="","",IFERROR(E19/INDEX(Paramètres!$E$4:$E$7,MATCH(D19,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
@@ -2486,7 +2823,7 @@
       <c r="B20" s="13"/>
       <c r="C20" s="13"/>
       <c r="D20" s="13"/>
-      <c r="E20" s="16"/>
+      <c r="E20" s="18"/>
       <c r="F20" s="6" t="str">
         <f aca="false">IF(A20="","",IFERROR(E20/INDEX(Paramètres!$E$4:$E$7,MATCH(D20,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
@@ -2514,7 +2851,7 @@
       <c r="B21" s="13"/>
       <c r="C21" s="13"/>
       <c r="D21" s="13"/>
-      <c r="E21" s="16"/>
+      <c r="E21" s="18"/>
       <c r="F21" s="6" t="str">
         <f aca="false">IF(A21="","",IFERROR(E21/INDEX(Paramètres!$E$4:$E$7,MATCH(D21,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
@@ -2542,7 +2879,7 @@
       <c r="B22" s="13"/>
       <c r="C22" s="13"/>
       <c r="D22" s="13"/>
-      <c r="E22" s="16"/>
+      <c r="E22" s="18"/>
       <c r="F22" s="6" t="str">
         <f aca="false">IF(A22="","",IFERROR(E22/INDEX(Paramètres!$E$4:$E$7,MATCH(D22,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
@@ -2570,7 +2907,7 @@
       <c r="B23" s="13"/>
       <c r="C23" s="13"/>
       <c r="D23" s="13"/>
-      <c r="E23" s="16"/>
+      <c r="E23" s="18"/>
       <c r="F23" s="6" t="str">
         <f aca="false">IF(A23="","",IFERROR(E23/INDEX(Paramètres!$E$4:$E$7,MATCH(D23,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
@@ -2598,7 +2935,7 @@
       <c r="B24" s="13"/>
       <c r="C24" s="13"/>
       <c r="D24" s="13"/>
-      <c r="E24" s="16"/>
+      <c r="E24" s="18"/>
       <c r="F24" s="6" t="str">
         <f aca="false">IF(A24="","",IFERROR(E24/INDEX(Paramètres!$E$4:$E$7,MATCH(D24,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
@@ -2626,7 +2963,7 @@
       <c r="B25" s="13"/>
       <c r="C25" s="13"/>
       <c r="D25" s="13"/>
-      <c r="E25" s="16"/>
+      <c r="E25" s="18"/>
       <c r="F25" s="6" t="str">
         <f aca="false">IF(A25="","",IFERROR(E25/INDEX(Paramètres!$E$4:$E$7,MATCH(D25,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
@@ -2654,7 +2991,7 @@
       <c r="B26" s="13"/>
       <c r="C26" s="13"/>
       <c r="D26" s="13"/>
-      <c r="E26" s="16"/>
+      <c r="E26" s="18"/>
       <c r="F26" s="6" t="str">
         <f aca="false">IF(A26="","",IFERROR(E26/INDEX(Paramètres!$E$4:$E$7,MATCH(D26,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
@@ -2682,7 +3019,7 @@
       <c r="B27" s="13"/>
       <c r="C27" s="13"/>
       <c r="D27" s="13"/>
-      <c r="E27" s="16"/>
+      <c r="E27" s="18"/>
       <c r="F27" s="6" t="str">
         <f aca="false">IF(A27="","",IFERROR(E27/INDEX(Paramètres!$E$4:$E$7,MATCH(D27,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
@@ -2710,7 +3047,7 @@
       <c r="B28" s="13"/>
       <c r="C28" s="13"/>
       <c r="D28" s="13"/>
-      <c r="E28" s="16"/>
+      <c r="E28" s="18"/>
       <c r="F28" s="6" t="str">
         <f aca="false">IF(A28="","",IFERROR(E28/INDEX(Paramètres!$E$4:$E$7,MATCH(D28,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
@@ -2738,7 +3075,7 @@
       <c r="B29" s="13"/>
       <c r="C29" s="13"/>
       <c r="D29" s="13"/>
-      <c r="E29" s="16"/>
+      <c r="E29" s="18"/>
       <c r="F29" s="6" t="str">
         <f aca="false">IF(A29="","",IFERROR(E29/INDEX(Paramètres!$E$4:$E$7,MATCH(D29,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
@@ -2766,7 +3103,7 @@
       <c r="B30" s="13"/>
       <c r="C30" s="13"/>
       <c r="D30" s="13"/>
-      <c r="E30" s="16"/>
+      <c r="E30" s="18"/>
       <c r="F30" s="6" t="str">
         <f aca="false">IF(A30="","",IFERROR(E30/INDEX(Paramètres!$E$4:$E$7,MATCH(D30,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
@@ -2794,7 +3131,7 @@
       <c r="B31" s="13"/>
       <c r="C31" s="13"/>
       <c r="D31" s="13"/>
-      <c r="E31" s="16"/>
+      <c r="E31" s="18"/>
       <c r="F31" s="6" t="str">
         <f aca="false">IF(A31="","",IFERROR(E31/INDEX(Paramètres!$E$4:$E$7,MATCH(D31,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
@@ -2822,7 +3159,7 @@
       <c r="B32" s="13"/>
       <c r="C32" s="13"/>
       <c r="D32" s="13"/>
-      <c r="E32" s="16"/>
+      <c r="E32" s="18"/>
       <c r="F32" s="6" t="str">
         <f aca="false">IF(A32="","",IFERROR(E32/INDEX(Paramètres!$E$4:$E$7,MATCH(D32,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
@@ -2850,7 +3187,7 @@
       <c r="B33" s="13"/>
       <c r="C33" s="13"/>
       <c r="D33" s="13"/>
-      <c r="E33" s="16"/>
+      <c r="E33" s="18"/>
       <c r="F33" s="6" t="str">
         <f aca="false">IF(A33="","",IFERROR(E33/INDEX(Paramètres!$E$4:$E$7,MATCH(D33,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
@@ -2878,7 +3215,7 @@
       <c r="B34" s="13"/>
       <c r="C34" s="13"/>
       <c r="D34" s="13"/>
-      <c r="E34" s="16"/>
+      <c r="E34" s="18"/>
       <c r="F34" s="6" t="str">
         <f aca="false">IF(A34="","",IFERROR(E34/INDEX(Paramètres!$E$4:$E$7,MATCH(D34,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
@@ -2906,7 +3243,7 @@
       <c r="B35" s="13"/>
       <c r="C35" s="13"/>
       <c r="D35" s="13"/>
-      <c r="E35" s="16"/>
+      <c r="E35" s="18"/>
       <c r="F35" s="6" t="str">
         <f aca="false">IF(A35="","",IFERROR(E35/INDEX(Paramètres!$E$4:$E$7,MATCH(D35,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
@@ -2934,7 +3271,7 @@
       <c r="B36" s="13"/>
       <c r="C36" s="13"/>
       <c r="D36" s="13"/>
-      <c r="E36" s="16"/>
+      <c r="E36" s="18"/>
       <c r="F36" s="6" t="str">
         <f aca="false">IF(A36="","",IFERROR(E36/INDEX(Paramètres!$E$4:$E$7,MATCH(D36,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
@@ -2962,7 +3299,7 @@
       <c r="B37" s="13"/>
       <c r="C37" s="13"/>
       <c r="D37" s="13"/>
-      <c r="E37" s="16"/>
+      <c r="E37" s="18"/>
       <c r="F37" s="6" t="str">
         <f aca="false">IF(A37="","",IFERROR(E37/INDEX(Paramètres!$E$4:$E$7,MATCH(D37,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
@@ -2990,7 +3327,7 @@
       <c r="B38" s="13"/>
       <c r="C38" s="13"/>
       <c r="D38" s="13"/>
-      <c r="E38" s="16"/>
+      <c r="E38" s="18"/>
       <c r="F38" s="6" t="str">
         <f aca="false">IF(A38="","",IFERROR(E38/INDEX(Paramètres!$E$4:$E$7,MATCH(D38,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
@@ -3018,7 +3355,7 @@
       <c r="B39" s="13"/>
       <c r="C39" s="13"/>
       <c r="D39" s="13"/>
-      <c r="E39" s="16"/>
+      <c r="E39" s="18"/>
       <c r="F39" s="6" t="str">
         <f aca="false">IF(A39="","",IFERROR(E39/INDEX(Paramètres!$E$4:$E$7,MATCH(D39,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
@@ -3046,7 +3383,7 @@
       <c r="B40" s="13"/>
       <c r="C40" s="13"/>
       <c r="D40" s="13"/>
-      <c r="E40" s="16"/>
+      <c r="E40" s="18"/>
       <c r="F40" s="6" t="str">
         <f aca="false">IF(A40="","",IFERROR(E40/INDEX(Paramètres!$E$4:$E$7,MATCH(D40,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
@@ -3074,7 +3411,7 @@
       <c r="B41" s="13"/>
       <c r="C41" s="13"/>
       <c r="D41" s="13"/>
-      <c r="E41" s="16"/>
+      <c r="E41" s="18"/>
       <c r="F41" s="6" t="str">
         <f aca="false">IF(A41="","",IFERROR(E41/INDEX(Paramètres!$E$4:$E$7,MATCH(D41,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
@@ -3102,7 +3439,7 @@
       <c r="B42" s="13"/>
       <c r="C42" s="13"/>
       <c r="D42" s="13"/>
-      <c r="E42" s="16"/>
+      <c r="E42" s="18"/>
       <c r="F42" s="6" t="str">
         <f aca="false">IF(A42="","",IFERROR(E42/INDEX(Paramètres!$E$4:$E$7,MATCH(D42,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
@@ -3130,7 +3467,7 @@
       <c r="B43" s="13"/>
       <c r="C43" s="13"/>
       <c r="D43" s="13"/>
-      <c r="E43" s="16"/>
+      <c r="E43" s="18"/>
       <c r="F43" s="6" t="str">
         <f aca="false">IF(A43="","",IFERROR(E43/INDEX(Paramètres!$E$4:$E$7,MATCH(D43,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
@@ -3158,7 +3495,7 @@
       <c r="B44" s="13"/>
       <c r="C44" s="13"/>
       <c r="D44" s="13"/>
-      <c r="E44" s="16"/>
+      <c r="E44" s="18"/>
       <c r="F44" s="6" t="str">
         <f aca="false">IF(A44="","",IFERROR(E44/INDEX(Paramètres!$E$4:$E$7,MATCH(D44,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
@@ -3186,7 +3523,7 @@
       <c r="B45" s="13"/>
       <c r="C45" s="13"/>
       <c r="D45" s="13"/>
-      <c r="E45" s="16"/>
+      <c r="E45" s="18"/>
       <c r="F45" s="6" t="str">
         <f aca="false">IF(A45="","",IFERROR(E45/INDEX(Paramètres!$E$4:$E$7,MATCH(D45,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
@@ -3214,7 +3551,7 @@
       <c r="B46" s="13"/>
       <c r="C46" s="13"/>
       <c r="D46" s="13"/>
-      <c r="E46" s="16"/>
+      <c r="E46" s="18"/>
       <c r="F46" s="6" t="str">
         <f aca="false">IF(A46="","",IFERROR(E46/INDEX(Paramètres!$E$4:$E$7,MATCH(D46,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
@@ -3242,7 +3579,7 @@
       <c r="B47" s="13"/>
       <c r="C47" s="13"/>
       <c r="D47" s="13"/>
-      <c r="E47" s="16"/>
+      <c r="E47" s="18"/>
       <c r="F47" s="6" t="str">
         <f aca="false">IF(A47="","",IFERROR(E47/INDEX(Paramètres!$E$4:$E$7,MATCH(D47,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
@@ -3270,7 +3607,7 @@
       <c r="B48" s="13"/>
       <c r="C48" s="13"/>
       <c r="D48" s="13"/>
-      <c r="E48" s="16"/>
+      <c r="E48" s="18"/>
       <c r="F48" s="6" t="str">
         <f aca="false">IF(A48="","",IFERROR(E48/INDEX(Paramètres!$E$4:$E$7,MATCH(D48,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
@@ -3298,7 +3635,7 @@
       <c r="B49" s="13"/>
       <c r="C49" s="13"/>
       <c r="D49" s="13"/>
-      <c r="E49" s="16"/>
+      <c r="E49" s="18"/>
       <c r="F49" s="6" t="str">
         <f aca="false">IF(A49="","",IFERROR(E49/INDEX(Paramètres!$E$4:$E$7,MATCH(D49,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
@@ -3326,7 +3663,7 @@
       <c r="B50" s="13"/>
       <c r="C50" s="13"/>
       <c r="D50" s="13"/>
-      <c r="E50" s="16"/>
+      <c r="E50" s="18"/>
       <c r="F50" s="6" t="str">
         <f aca="false">IF(A50="","",IFERROR(E50/INDEX(Paramètres!$E$4:$E$7,MATCH(D50,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
@@ -3354,7 +3691,7 @@
       <c r="B51" s="13"/>
       <c r="C51" s="13"/>
       <c r="D51" s="13"/>
-      <c r="E51" s="16"/>
+      <c r="E51" s="18"/>
       <c r="F51" s="6" t="str">
         <f aca="false">IF(A51="","",IFERROR(E51/INDEX(Paramètres!$E$4:$E$7,MATCH(D51,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
@@ -3382,7 +3719,7 @@
       <c r="B52" s="13"/>
       <c r="C52" s="13"/>
       <c r="D52" s="13"/>
-      <c r="E52" s="16"/>
+      <c r="E52" s="18"/>
       <c r="F52" s="6" t="str">
         <f aca="false">IF(A52="","",IFERROR(E52/INDEX(Paramètres!$E$4:$E$7,MATCH(D52,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
@@ -3410,7 +3747,7 @@
       <c r="B53" s="13"/>
       <c r="C53" s="13"/>
       <c r="D53" s="13"/>
-      <c r="E53" s="16"/>
+      <c r="E53" s="18"/>
       <c r="F53" s="6" t="str">
         <f aca="false">IF(A53="","",IFERROR(E53/INDEX(Paramètres!$E$4:$E$7,MATCH(D53,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
@@ -3438,7 +3775,7 @@
       <c r="B54" s="13"/>
       <c r="C54" s="13"/>
       <c r="D54" s="13"/>
-      <c r="E54" s="16"/>
+      <c r="E54" s="18"/>
       <c r="F54" s="6" t="str">
         <f aca="false">IF(A54="","",IFERROR(E54/INDEX(Paramètres!$E$4:$E$7,MATCH(D54,Paramètres!$D$4:$D$7,0)),0))</f>
         <v/>
@@ -3462,20 +3799,20 @@
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="17" t="s">
-        <v>100</v>
+      <c r="A55" s="20" t="s">
+        <v>122</v>
       </c>
       <c r="F55" s="9" t="n">
         <f aca="false">SUM(F5:F54)</f>
-        <v>2401.33333333333</v>
+        <v>2523</v>
       </c>
       <c r="M55" s="9" t="n">
         <f aca="false">SUM(M5:M54)</f>
-        <v>1294.82558139535</v>
+        <v>1355.65891472868</v>
       </c>
       <c r="N55" s="9" t="n">
         <f aca="false">SUM(N5:N54)</f>
-        <v>1106.50775193798</v>
+        <v>1167.34108527132</v>
       </c>
     </row>
   </sheetData>
@@ -3530,62 +3867,62 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>101</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>102</v>
+        <v>124</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>63</v>
+        <v>81</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>3</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>67</v>
+        <v>85</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>103</v>
+        <v>125</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>71</v>
+        <v>89</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>104</v>
+        <v>126</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>105</v>
+        <v>127</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="D5" s="16" t="n">
+        <v>35</v>
+      </c>
+      <c r="D5" s="18" t="n">
         <v>2400</v>
       </c>
       <c r="E5" s="13" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="F5" s="6" t="n">
         <f aca="false">IF(A5="","",IFERROR(D5/INDEX(Paramètres!$E$4:$E$7,MATCH(E5,Paramètres!$D$4:$D$7,0)),0))</f>
         <v>2400</v>
       </c>
       <c r="G5" s="13" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="H5" s="13" t="n">
         <v>28</v>
@@ -3593,26 +3930,26 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>106</v>
+        <v>128</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>105</v>
+        <v>127</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="D6" s="16" t="n">
+        <v>38</v>
+      </c>
+      <c r="D6" s="18" t="n">
         <v>1900</v>
       </c>
       <c r="E6" s="13" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="F6" s="6" t="n">
         <f aca="false">IF(A6="","",IFERROR(D6/INDEX(Paramètres!$E$4:$E$7,MATCH(E6,Paramètres!$D$4:$D$7,0)),0))</f>
         <v>1900</v>
       </c>
       <c r="G6" s="13" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="H6" s="13" t="n">
         <v>30</v>
@@ -3620,26 +3957,26 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>107</v>
+        <v>129</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>108</v>
+        <v>130</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>109</v>
-      </c>
-      <c r="D7" s="16" t="n">
+        <v>131</v>
+      </c>
+      <c r="D7" s="18" t="n">
         <v>140</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="F7" s="6" t="n">
         <f aca="false">IF(A7="","",IFERROR(D7/INDEX(Paramètres!$E$4:$E$7,MATCH(E7,Paramètres!$D$4:$D$7,0)),0))</f>
         <v>140</v>
       </c>
       <c r="G7" s="13" t="s">
-        <v>54</v>
+        <v>72</v>
       </c>
       <c r="H7" s="13" t="n">
         <v>5</v>
@@ -3647,26 +3984,26 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>110</v>
+        <v>132</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>108</v>
+        <v>130</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>109</v>
-      </c>
-      <c r="D8" s="16" t="n">
+        <v>131</v>
+      </c>
+      <c r="D8" s="18" t="n">
         <v>270</v>
       </c>
       <c r="E8" s="13" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="F8" s="6" t="n">
         <f aca="false">IF(A8="","",IFERROR(D8/INDEX(Paramètres!$E$4:$E$7,MATCH(E8,Paramètres!$D$4:$D$7,0)),0))</f>
         <v>90</v>
       </c>
       <c r="G8" s="13" t="s">
-        <v>54</v>
+        <v>72</v>
       </c>
       <c r="H8" s="13" t="n">
         <v>5</v>
@@ -3676,7 +4013,7 @@
       <c r="A9" s="13"/>
       <c r="B9" s="13"/>
       <c r="C9" s="13"/>
-      <c r="D9" s="16"/>
+      <c r="D9" s="18"/>
       <c r="E9" s="13"/>
       <c r="F9" s="6" t="str">
         <f aca="false">IF(A9="","",IFERROR(D9/INDEX(Paramètres!$E$4:$E$7,MATCH(E9,Paramètres!$D$4:$D$7,0)),0))</f>
@@ -3689,7 +4026,7 @@
       <c r="A10" s="13"/>
       <c r="B10" s="13"/>
       <c r="C10" s="13"/>
-      <c r="D10" s="16"/>
+      <c r="D10" s="18"/>
       <c r="E10" s="13"/>
       <c r="F10" s="6" t="str">
         <f aca="false">IF(A10="","",IFERROR(D10/INDEX(Paramètres!$E$4:$E$7,MATCH(E10,Paramètres!$D$4:$D$7,0)),0))</f>
@@ -3702,7 +4039,7 @@
       <c r="A11" s="13"/>
       <c r="B11" s="13"/>
       <c r="C11" s="13"/>
-      <c r="D11" s="16"/>
+      <c r="D11" s="18"/>
       <c r="E11" s="13"/>
       <c r="F11" s="6" t="str">
         <f aca="false">IF(A11="","",IFERROR(D11/INDEX(Paramètres!$E$4:$E$7,MATCH(E11,Paramètres!$D$4:$D$7,0)),0))</f>
@@ -3715,7 +4052,7 @@
       <c r="A12" s="13"/>
       <c r="B12" s="13"/>
       <c r="C12" s="13"/>
-      <c r="D12" s="16"/>
+      <c r="D12" s="18"/>
       <c r="E12" s="13"/>
       <c r="F12" s="6" t="str">
         <f aca="false">IF(A12="","",IFERROR(D12/INDEX(Paramètres!$E$4:$E$7,MATCH(E12,Paramètres!$D$4:$D$7,0)),0))</f>
@@ -3728,7 +4065,7 @@
       <c r="A13" s="13"/>
       <c r="B13" s="13"/>
       <c r="C13" s="13"/>
-      <c r="D13" s="16"/>
+      <c r="D13" s="18"/>
       <c r="E13" s="13"/>
       <c r="F13" s="6" t="str">
         <f aca="false">IF(A13="","",IFERROR(D13/INDEX(Paramètres!$E$4:$E$7,MATCH(E13,Paramètres!$D$4:$D$7,0)),0))</f>
@@ -3741,7 +4078,7 @@
       <c r="A14" s="13"/>
       <c r="B14" s="13"/>
       <c r="C14" s="13"/>
-      <c r="D14" s="16"/>
+      <c r="D14" s="18"/>
       <c r="E14" s="13"/>
       <c r="F14" s="6" t="str">
         <f aca="false">IF(A14="","",IFERROR(D14/INDEX(Paramètres!$E$4:$E$7,MATCH(E14,Paramètres!$D$4:$D$7,0)),0))</f>
@@ -3754,7 +4091,7 @@
       <c r="A15" s="13"/>
       <c r="B15" s="13"/>
       <c r="C15" s="13"/>
-      <c r="D15" s="16"/>
+      <c r="D15" s="18"/>
       <c r="E15" s="13"/>
       <c r="F15" s="6" t="str">
         <f aca="false">IF(A15="","",IFERROR(D15/INDEX(Paramètres!$E$4:$E$7,MATCH(E15,Paramètres!$D$4:$D$7,0)),0))</f>
@@ -3767,7 +4104,7 @@
       <c r="A16" s="13"/>
       <c r="B16" s="13"/>
       <c r="C16" s="13"/>
-      <c r="D16" s="16"/>
+      <c r="D16" s="18"/>
       <c r="E16" s="13"/>
       <c r="F16" s="6" t="str">
         <f aca="false">IF(A16="","",IFERROR(D16/INDEX(Paramètres!$E$4:$E$7,MATCH(E16,Paramètres!$D$4:$D$7,0)),0))</f>
@@ -3780,7 +4117,7 @@
       <c r="A17" s="13"/>
       <c r="B17" s="13"/>
       <c r="C17" s="13"/>
-      <c r="D17" s="16"/>
+      <c r="D17" s="18"/>
       <c r="E17" s="13"/>
       <c r="F17" s="6" t="str">
         <f aca="false">IF(A17="","",IFERROR(D17/INDEX(Paramètres!$E$4:$E$7,MATCH(E17,Paramètres!$D$4:$D$7,0)),0))</f>
@@ -3793,7 +4130,7 @@
       <c r="A18" s="13"/>
       <c r="B18" s="13"/>
       <c r="C18" s="13"/>
-      <c r="D18" s="16"/>
+      <c r="D18" s="18"/>
       <c r="E18" s="13"/>
       <c r="F18" s="6" t="str">
         <f aca="false">IF(A18="","",IFERROR(D18/INDEX(Paramètres!$E$4:$E$7,MATCH(E18,Paramètres!$D$4:$D$7,0)),0))</f>
@@ -3806,7 +4143,7 @@
       <c r="A19" s="13"/>
       <c r="B19" s="13"/>
       <c r="C19" s="13"/>
-      <c r="D19" s="16"/>
+      <c r="D19" s="18"/>
       <c r="E19" s="13"/>
       <c r="F19" s="6" t="str">
         <f aca="false">IF(A19="","",IFERROR(D19/INDEX(Paramètres!$E$4:$E$7,MATCH(E19,Paramètres!$D$4:$D$7,0)),0))</f>
@@ -3819,7 +4156,7 @@
       <c r="A20" s="13"/>
       <c r="B20" s="13"/>
       <c r="C20" s="13"/>
-      <c r="D20" s="16"/>
+      <c r="D20" s="18"/>
       <c r="E20" s="13"/>
       <c r="F20" s="6" t="str">
         <f aca="false">IF(A20="","",IFERROR(D20/INDEX(Paramètres!$E$4:$E$7,MATCH(E20,Paramètres!$D$4:$D$7,0)),0))</f>
@@ -3832,7 +4169,7 @@
       <c r="A21" s="13"/>
       <c r="B21" s="13"/>
       <c r="C21" s="13"/>
-      <c r="D21" s="16"/>
+      <c r="D21" s="18"/>
       <c r="E21" s="13"/>
       <c r="F21" s="6" t="str">
         <f aca="false">IF(A21="","",IFERROR(D21/INDEX(Paramètres!$E$4:$E$7,MATCH(E21,Paramètres!$D$4:$D$7,0)),0))</f>
@@ -3845,7 +4182,7 @@
       <c r="A22" s="13"/>
       <c r="B22" s="13"/>
       <c r="C22" s="13"/>
-      <c r="D22" s="16"/>
+      <c r="D22" s="18"/>
       <c r="E22" s="13"/>
       <c r="F22" s="6" t="str">
         <f aca="false">IF(A22="","",IFERROR(D22/INDEX(Paramètres!$E$4:$E$7,MATCH(E22,Paramètres!$D$4:$D$7,0)),0))</f>
@@ -3858,7 +4195,7 @@
       <c r="A23" s="13"/>
       <c r="B23" s="13"/>
       <c r="C23" s="13"/>
-      <c r="D23" s="16"/>
+      <c r="D23" s="18"/>
       <c r="E23" s="13"/>
       <c r="F23" s="6" t="str">
         <f aca="false">IF(A23="","",IFERROR(D23/INDEX(Paramètres!$E$4:$E$7,MATCH(E23,Paramètres!$D$4:$D$7,0)),0))</f>
@@ -3871,7 +4208,7 @@
       <c r="A24" s="13"/>
       <c r="B24" s="13"/>
       <c r="C24" s="13"/>
-      <c r="D24" s="16"/>
+      <c r="D24" s="18"/>
       <c r="E24" s="13"/>
       <c r="F24" s="6" t="str">
         <f aca="false">IF(A24="","",IFERROR(D24/INDEX(Paramètres!$E$4:$E$7,MATCH(E24,Paramètres!$D$4:$D$7,0)),0))</f>
@@ -3881,8 +4218,8 @@
       <c r="H24" s="13"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="17" t="s">
-        <v>100</v>
+      <c r="A25" s="20" t="s">
+        <v>122</v>
       </c>
       <c r="F25" s="9" t="n">
         <f aca="false">SUM(F5:F24)</f>
@@ -3912,4 +4249,548 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:F45"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="13" t="s">
+        <v>135</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>121</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="E5" s="18" t="n">
+        <v>35</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <f aca="false">IF(A5="","",IFERROR(E5/INDEX(Paramètres!$E$4:$E$7,MATCH(D5,Paramètres!$D$4:$D$7,0)),0))</f>
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="13" t="s">
+        <v>136</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>137</v>
+      </c>
+      <c r="D6" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="E6" s="18" t="n">
+        <v>120</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <f aca="false">IF(A6="","",IFERROR(E6/INDEX(Paramètres!$E$4:$E$7,MATCH(D6,Paramètres!$D$4:$D$7,0)),0))</f>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="13" t="s">
+        <v>138</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="D7" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="E7" s="18" t="n">
+        <v>11</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <f aca="false">IF(A7="","",IFERROR(E7/INDEX(Paramètres!$E$4:$E$7,MATCH(D7,Paramètres!$D$4:$D$7,0)),0))</f>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="13"/>
+      <c r="B8" s="13"/>
+      <c r="C8" s="13"/>
+      <c r="D8" s="13"/>
+      <c r="E8" s="18"/>
+      <c r="F8" s="6" t="str">
+        <f aca="false">IF(A8="","",IFERROR(E8/INDEX(Paramètres!$E$4:$E$7,MATCH(D8,Paramètres!$D$4:$D$7,0)),0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="13"/>
+      <c r="B9" s="13"/>
+      <c r="C9" s="13"/>
+      <c r="D9" s="13"/>
+      <c r="E9" s="18"/>
+      <c r="F9" s="6" t="str">
+        <f aca="false">IF(A9="","",IFERROR(E9/INDEX(Paramètres!$E$4:$E$7,MATCH(D9,Paramètres!$D$4:$D$7,0)),0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="13"/>
+      <c r="B10" s="13"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="13"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="6" t="str">
+        <f aca="false">IF(A10="","",IFERROR(E10/INDEX(Paramètres!$E$4:$E$7,MATCH(D10,Paramètres!$D$4:$D$7,0)),0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="13"/>
+      <c r="B11" s="13"/>
+      <c r="C11" s="13"/>
+      <c r="D11" s="13"/>
+      <c r="E11" s="18"/>
+      <c r="F11" s="6" t="str">
+        <f aca="false">IF(A11="","",IFERROR(E11/INDEX(Paramètres!$E$4:$E$7,MATCH(D11,Paramètres!$D$4:$D$7,0)),0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="13"/>
+      <c r="B12" s="13"/>
+      <c r="C12" s="13"/>
+      <c r="D12" s="13"/>
+      <c r="E12" s="18"/>
+      <c r="F12" s="6" t="str">
+        <f aca="false">IF(A12="","",IFERROR(E12/INDEX(Paramètres!$E$4:$E$7,MATCH(D12,Paramètres!$D$4:$D$7,0)),0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="13"/>
+      <c r="B13" s="13"/>
+      <c r="C13" s="13"/>
+      <c r="D13" s="13"/>
+      <c r="E13" s="18"/>
+      <c r="F13" s="6" t="str">
+        <f aca="false">IF(A13="","",IFERROR(E13/INDEX(Paramètres!$E$4:$E$7,MATCH(D13,Paramètres!$D$4:$D$7,0)),0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="13"/>
+      <c r="B14" s="13"/>
+      <c r="C14" s="13"/>
+      <c r="D14" s="13"/>
+      <c r="E14" s="18"/>
+      <c r="F14" s="6" t="str">
+        <f aca="false">IF(A14="","",IFERROR(E14/INDEX(Paramètres!$E$4:$E$7,MATCH(D14,Paramètres!$D$4:$D$7,0)),0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="13"/>
+      <c r="B15" s="13"/>
+      <c r="C15" s="13"/>
+      <c r="D15" s="13"/>
+      <c r="E15" s="18"/>
+      <c r="F15" s="6" t="str">
+        <f aca="false">IF(A15="","",IFERROR(E15/INDEX(Paramètres!$E$4:$E$7,MATCH(D15,Paramètres!$D$4:$D$7,0)),0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="13"/>
+      <c r="B16" s="13"/>
+      <c r="C16" s="13"/>
+      <c r="D16" s="13"/>
+      <c r="E16" s="18"/>
+      <c r="F16" s="6" t="str">
+        <f aca="false">IF(A16="","",IFERROR(E16/INDEX(Paramètres!$E$4:$E$7,MATCH(D16,Paramètres!$D$4:$D$7,0)),0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="13"/>
+      <c r="B17" s="13"/>
+      <c r="C17" s="13"/>
+      <c r="D17" s="13"/>
+      <c r="E17" s="18"/>
+      <c r="F17" s="6" t="str">
+        <f aca="false">IF(A17="","",IFERROR(E17/INDEX(Paramètres!$E$4:$E$7,MATCH(D17,Paramètres!$D$4:$D$7,0)),0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="13"/>
+      <c r="B18" s="13"/>
+      <c r="C18" s="13"/>
+      <c r="D18" s="13"/>
+      <c r="E18" s="18"/>
+      <c r="F18" s="6" t="str">
+        <f aca="false">IF(A18="","",IFERROR(E18/INDEX(Paramètres!$E$4:$E$7,MATCH(D18,Paramètres!$D$4:$D$7,0)),0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="13"/>
+      <c r="B19" s="13"/>
+      <c r="C19" s="13"/>
+      <c r="D19" s="13"/>
+      <c r="E19" s="18"/>
+      <c r="F19" s="6" t="str">
+        <f aca="false">IF(A19="","",IFERROR(E19/INDEX(Paramètres!$E$4:$E$7,MATCH(D19,Paramètres!$D$4:$D$7,0)),0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="13"/>
+      <c r="B20" s="13"/>
+      <c r="C20" s="13"/>
+      <c r="D20" s="13"/>
+      <c r="E20" s="18"/>
+      <c r="F20" s="6" t="str">
+        <f aca="false">IF(A20="","",IFERROR(E20/INDEX(Paramètres!$E$4:$E$7,MATCH(D20,Paramètres!$D$4:$D$7,0)),0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="13"/>
+      <c r="B21" s="13"/>
+      <c r="C21" s="13"/>
+      <c r="D21" s="13"/>
+      <c r="E21" s="18"/>
+      <c r="F21" s="6" t="str">
+        <f aca="false">IF(A21="","",IFERROR(E21/INDEX(Paramètres!$E$4:$E$7,MATCH(D21,Paramètres!$D$4:$D$7,0)),0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="13"/>
+      <c r="B22" s="13"/>
+      <c r="C22" s="13"/>
+      <c r="D22" s="13"/>
+      <c r="E22" s="18"/>
+      <c r="F22" s="6" t="str">
+        <f aca="false">IF(A22="","",IFERROR(E22/INDEX(Paramètres!$E$4:$E$7,MATCH(D22,Paramètres!$D$4:$D$7,0)),0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="13"/>
+      <c r="B23" s="13"/>
+      <c r="C23" s="13"/>
+      <c r="D23" s="13"/>
+      <c r="E23" s="18"/>
+      <c r="F23" s="6" t="str">
+        <f aca="false">IF(A23="","",IFERROR(E23/INDEX(Paramètres!$E$4:$E$7,MATCH(D23,Paramètres!$D$4:$D$7,0)),0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="13"/>
+      <c r="B24" s="13"/>
+      <c r="C24" s="13"/>
+      <c r="D24" s="13"/>
+      <c r="E24" s="18"/>
+      <c r="F24" s="6" t="str">
+        <f aca="false">IF(A24="","",IFERROR(E24/INDEX(Paramètres!$E$4:$E$7,MATCH(D24,Paramètres!$D$4:$D$7,0)),0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="13"/>
+      <c r="B25" s="13"/>
+      <c r="C25" s="13"/>
+      <c r="D25" s="13"/>
+      <c r="E25" s="18"/>
+      <c r="F25" s="6" t="str">
+        <f aca="false">IF(A25="","",IFERROR(E25/INDEX(Paramètres!$E$4:$E$7,MATCH(D25,Paramètres!$D$4:$D$7,0)),0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="13"/>
+      <c r="B26" s="13"/>
+      <c r="C26" s="13"/>
+      <c r="D26" s="13"/>
+      <c r="E26" s="18"/>
+      <c r="F26" s="6" t="str">
+        <f aca="false">IF(A26="","",IFERROR(E26/INDEX(Paramètres!$E$4:$E$7,MATCH(D26,Paramètres!$D$4:$D$7,0)),0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="13"/>
+      <c r="B27" s="13"/>
+      <c r="C27" s="13"/>
+      <c r="D27" s="13"/>
+      <c r="E27" s="18"/>
+      <c r="F27" s="6" t="str">
+        <f aca="false">IF(A27="","",IFERROR(E27/INDEX(Paramètres!$E$4:$E$7,MATCH(D27,Paramètres!$D$4:$D$7,0)),0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="13"/>
+      <c r="B28" s="13"/>
+      <c r="C28" s="13"/>
+      <c r="D28" s="13"/>
+      <c r="E28" s="18"/>
+      <c r="F28" s="6" t="str">
+        <f aca="false">IF(A28="","",IFERROR(E28/INDEX(Paramètres!$E$4:$E$7,MATCH(D28,Paramètres!$D$4:$D$7,0)),0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="13"/>
+      <c r="B29" s="13"/>
+      <c r="C29" s="13"/>
+      <c r="D29" s="13"/>
+      <c r="E29" s="18"/>
+      <c r="F29" s="6" t="str">
+        <f aca="false">IF(A29="","",IFERROR(E29/INDEX(Paramètres!$E$4:$E$7,MATCH(D29,Paramètres!$D$4:$D$7,0)),0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="13"/>
+      <c r="B30" s="13"/>
+      <c r="C30" s="13"/>
+      <c r="D30" s="13"/>
+      <c r="E30" s="18"/>
+      <c r="F30" s="6" t="str">
+        <f aca="false">IF(A30="","",IFERROR(E30/INDEX(Paramètres!$E$4:$E$7,MATCH(D30,Paramètres!$D$4:$D$7,0)),0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="13"/>
+      <c r="B31" s="13"/>
+      <c r="C31" s="13"/>
+      <c r="D31" s="13"/>
+      <c r="E31" s="18"/>
+      <c r="F31" s="6" t="str">
+        <f aca="false">IF(A31="","",IFERROR(E31/INDEX(Paramètres!$E$4:$E$7,MATCH(D31,Paramètres!$D$4:$D$7,0)),0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="13"/>
+      <c r="B32" s="13"/>
+      <c r="C32" s="13"/>
+      <c r="D32" s="13"/>
+      <c r="E32" s="18"/>
+      <c r="F32" s="6" t="str">
+        <f aca="false">IF(A32="","",IFERROR(E32/INDEX(Paramètres!$E$4:$E$7,MATCH(D32,Paramètres!$D$4:$D$7,0)),0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="13"/>
+      <c r="B33" s="13"/>
+      <c r="C33" s="13"/>
+      <c r="D33" s="13"/>
+      <c r="E33" s="18"/>
+      <c r="F33" s="6" t="str">
+        <f aca="false">IF(A33="","",IFERROR(E33/INDEX(Paramètres!$E$4:$E$7,MATCH(D33,Paramètres!$D$4:$D$7,0)),0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="13"/>
+      <c r="B34" s="13"/>
+      <c r="C34" s="13"/>
+      <c r="D34" s="13"/>
+      <c r="E34" s="18"/>
+      <c r="F34" s="6" t="str">
+        <f aca="false">IF(A34="","",IFERROR(E34/INDEX(Paramètres!$E$4:$E$7,MATCH(D34,Paramètres!$D$4:$D$7,0)),0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="13"/>
+      <c r="B35" s="13"/>
+      <c r="C35" s="13"/>
+      <c r="D35" s="13"/>
+      <c r="E35" s="18"/>
+      <c r="F35" s="6" t="str">
+        <f aca="false">IF(A35="","",IFERROR(E35/INDEX(Paramètres!$E$4:$E$7,MATCH(D35,Paramètres!$D$4:$D$7,0)),0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="13"/>
+      <c r="B36" s="13"/>
+      <c r="C36" s="13"/>
+      <c r="D36" s="13"/>
+      <c r="E36" s="18"/>
+      <c r="F36" s="6" t="str">
+        <f aca="false">IF(A36="","",IFERROR(E36/INDEX(Paramètres!$E$4:$E$7,MATCH(D36,Paramètres!$D$4:$D$7,0)),0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="13"/>
+      <c r="B37" s="13"/>
+      <c r="C37" s="13"/>
+      <c r="D37" s="13"/>
+      <c r="E37" s="18"/>
+      <c r="F37" s="6" t="str">
+        <f aca="false">IF(A37="","",IFERROR(E37/INDEX(Paramètres!$E$4:$E$7,MATCH(D37,Paramètres!$D$4:$D$7,0)),0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="13"/>
+      <c r="B38" s="13"/>
+      <c r="C38" s="13"/>
+      <c r="D38" s="13"/>
+      <c r="E38" s="18"/>
+      <c r="F38" s="6" t="str">
+        <f aca="false">IF(A38="","",IFERROR(E38/INDEX(Paramètres!$E$4:$E$7,MATCH(D38,Paramètres!$D$4:$D$7,0)),0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="13"/>
+      <c r="B39" s="13"/>
+      <c r="C39" s="13"/>
+      <c r="D39" s="13"/>
+      <c r="E39" s="18"/>
+      <c r="F39" s="6" t="str">
+        <f aca="false">IF(A39="","",IFERROR(E39/INDEX(Paramètres!$E$4:$E$7,MATCH(D39,Paramètres!$D$4:$D$7,0)),0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="13"/>
+      <c r="B40" s="13"/>
+      <c r="C40" s="13"/>
+      <c r="D40" s="13"/>
+      <c r="E40" s="18"/>
+      <c r="F40" s="6" t="str">
+        <f aca="false">IF(A40="","",IFERROR(E40/INDEX(Paramètres!$E$4:$E$7,MATCH(D40,Paramètres!$D$4:$D$7,0)),0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="13"/>
+      <c r="B41" s="13"/>
+      <c r="C41" s="13"/>
+      <c r="D41" s="13"/>
+      <c r="E41" s="18"/>
+      <c r="F41" s="6" t="str">
+        <f aca="false">IF(A41="","",IFERROR(E41/INDEX(Paramètres!$E$4:$E$7,MATCH(D41,Paramètres!$D$4:$D$7,0)),0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="13"/>
+      <c r="B42" s="13"/>
+      <c r="C42" s="13"/>
+      <c r="D42" s="13"/>
+      <c r="E42" s="18"/>
+      <c r="F42" s="6" t="str">
+        <f aca="false">IF(A42="","",IFERROR(E42/INDEX(Paramètres!$E$4:$E$7,MATCH(D42,Paramètres!$D$4:$D$7,0)),0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="13"/>
+      <c r="B43" s="13"/>
+      <c r="C43" s="13"/>
+      <c r="D43" s="13"/>
+      <c r="E43" s="18"/>
+      <c r="F43" s="6" t="str">
+        <f aca="false">IF(A43="","",IFERROR(E43/INDEX(Paramètres!$E$4:$E$7,MATCH(D43,Paramètres!$D$4:$D$7,0)),0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="13"/>
+      <c r="B44" s="13"/>
+      <c r="C44" s="13"/>
+      <c r="D44" s="13"/>
+      <c r="E44" s="18"/>
+      <c r="F44" s="6" t="str">
+        <f aca="false">IF(A44="","",IFERROR(E44/INDEX(Paramètres!$E$4:$E$7,MATCH(D44,Paramètres!$D$4:$D$7,0)),0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="20" t="s">
+        <v>122</v>
+      </c>
+      <c r="F45" s="9" t="n">
+        <f aca="false">SUM(F5:F44)</f>
+        <v>86</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="2">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D5:D44" type="list">
+      <formula1>"Mensuelle,Trimestrielle,Semestrielle,Annuelle"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B5:B44" type="list">
+      <formula1>Paramètres!$B$4:$B$5</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Ajout de la provision imprévus en pourcentage des salaires
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KqkJNWVZSWN9upSPoUaH5h
</commit_message>
<xml_diff>
--- a/suivi_comptes.xlsx
+++ b/suivi_comptes.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="143">
   <si>
     <t xml:space="preserve">Synthèse mensuelle</t>
   </si>
@@ -207,6 +207,12 @@
     <t xml:space="preserve">Si l'un de vous ne veut pas détailler ses comptes : mode Forfait + une somme. Ses lignes éventuelles dans « Charges perso » sont alors ignorées.</t>
   </si>
   <si>
+    <t xml:space="preserve">Provision imprévus (% des salaires du foyer)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alimente la ligne « Provision imprévus » de l'onglet Charges (réparties 50/50, sur le compte joint indiqué).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Comptes bancaires</t>
   </si>
   <si>
@@ -391,6 +397,12 @@
   </si>
   <si>
     <t xml:space="preserve">Loisirs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Provision imprévus (% des salaires)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Imprévus</t>
   </si>
   <si>
     <t xml:space="preserve">TOTAL mensuel</t>
@@ -627,7 +639,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -705,6 +717,14 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1038,7 +1058,7 @@
       </c>
       <c r="C5" s="6" t="n">
         <f aca="false">SUM(E$13:E$22)</f>
-        <v>1232.85600681269</v>
+        <v>1298.22324557302</v>
       </c>
       <c r="D5" s="6" t="n">
         <f aca="false">IFERROR(INDEX($C$13:$C$22,MATCH(Paramètres!$B$6,$A$13:$A$22,0)),0)</f>
@@ -1046,15 +1066,15 @@
       </c>
       <c r="E5" s="6" t="n">
         <f aca="false">C5+D5</f>
-        <v>1232.85600681269</v>
+        <v>1298.22324557302</v>
       </c>
       <c r="F5" s="7" t="n">
         <f aca="false">IF(B5=0,0,E5/B5)</f>
-        <v>0.51369000283862</v>
+        <v>0.540926352322094</v>
       </c>
       <c r="G5" s="6" t="n">
         <f aca="false">IFERROR(INDEX($J$13:$J$22,MATCH(Paramètres!$B$6,$A$13:$A$22,0)),0)</f>
-        <v>1167.14399318731</v>
+        <v>1101.77675442698</v>
       </c>
       <c r="H5" s="6" t="n">
         <f aca="false">IF(Paramètres!B$15="Forfait",Paramètres!B$16,SUMIFS('Charges perso'!$F$5:$F$44,'Charges perso'!$B$5:$B$44,A5))</f>
@@ -1062,15 +1082,15 @@
       </c>
       <c r="I5" s="6" t="n">
         <f aca="false">G5-H5</f>
-        <v>1081.14399318731</v>
+        <v>1015.77675442698</v>
       </c>
       <c r="J5" s="6" t="n">
         <f aca="false">MAX(0,IF(Paramètres!B$17="Pourcentage",Paramètres!B$18*MAX(0,I5),Paramètres!B$19))</f>
-        <v>324.343197956193</v>
+        <v>304.733026328093</v>
       </c>
       <c r="K5" s="6" t="n">
         <f aca="false">I5-J5</f>
-        <v>756.800795231118</v>
+        <v>711.043728098883</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1084,7 +1104,7 @@
       </c>
       <c r="C6" s="6" t="n">
         <f aca="false">SUM(F$13:F$22)</f>
-        <v>1032.14399318731</v>
+        <v>1095.77675442698</v>
       </c>
       <c r="D6" s="6" t="n">
         <f aca="false">IFERROR(INDEX($C$13:$C$22,MATCH(Paramètres!$B$7,$A$13:$A$22,0)),0)</f>
@@ -1092,15 +1112,15 @@
       </c>
       <c r="E6" s="6" t="n">
         <f aca="false">C6+D6</f>
-        <v>1060.14399318731</v>
+        <v>1123.77675442698</v>
       </c>
       <c r="F6" s="7" t="n">
         <f aca="false">IF(B6=0,0,E6/B6)</f>
-        <v>0.557970522730164</v>
+        <v>0.591461449698408</v>
       </c>
       <c r="G6" s="6" t="n">
         <f aca="false">IFERROR(INDEX($J$13:$J$22,MATCH(Paramètres!$B$7,$A$13:$A$22,0)),0)</f>
-        <v>839.856006812689</v>
+        <v>776.223245573025</v>
       </c>
       <c r="H6" s="6" t="n">
         <f aca="false">IF(Paramètres!C$15="Forfait",Paramètres!C$16,SUMIFS('Charges perso'!$F$5:$F$44,'Charges perso'!$B$5:$B$44,A6))</f>
@@ -1108,7 +1128,7 @@
       </c>
       <c r="I6" s="6" t="n">
         <f aca="false">G6-H6</f>
-        <v>489.856006812689</v>
+        <v>426.223245573025</v>
       </c>
       <c r="J6" s="6" t="n">
         <f aca="false">MAX(0,IF(Paramètres!C$17="Pourcentage",Paramètres!C$18*MAX(0,I6),Paramètres!C$19))</f>
@@ -1116,7 +1136,7 @@
       </c>
       <c r="K6" s="6" t="n">
         <f aca="false">I6-J6</f>
-        <v>289.856006812689</v>
+        <v>226.223245573025</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1129,7 +1149,7 @@
       </c>
       <c r="C7" s="9" t="n">
         <f aca="false">SUM(C5:C6)</f>
-        <v>2265</v>
+        <v>2394</v>
       </c>
       <c r="D7" s="9" t="n">
         <f aca="false">SUM(D5:D6)</f>
@@ -1137,15 +1157,15 @@
       </c>
       <c r="E7" s="9" t="n">
         <f aca="false">SUM(E5:E6)</f>
-        <v>2293</v>
+        <v>2422</v>
       </c>
       <c r="F7" s="10" t="n">
         <f aca="false">IF(B7=0,0,E7/B7)</f>
-        <v>0.533255813953488</v>
+        <v>0.563255813953488</v>
       </c>
       <c r="G7" s="9" t="n">
         <f aca="false">SUM(G5:G6)</f>
-        <v>2007</v>
+        <v>1878</v>
       </c>
       <c r="H7" s="9" t="n">
         <f aca="false">SUM(H5:H6)</f>
@@ -1153,15 +1173,15 @@
       </c>
       <c r="I7" s="9" t="n">
         <f aca="false">SUM(I5:I6)</f>
-        <v>1571</v>
+        <v>1442</v>
       </c>
       <c r="J7" s="9" t="n">
         <f aca="false">SUM(J5:J6)</f>
-        <v>524.343197956193</v>
+        <v>504.733026328093</v>
       </c>
       <c r="K7" s="9" t="n">
         <f aca="false">SUM(K5:K6)</f>
-        <v>1046.65680204381</v>
+        <v>937.266973671907</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1243,11 +1263,11 @@
       </c>
       <c r="I13" s="6" t="n">
         <f aca="false">IF($A13="","",IF($A13=Paramètres!$B$6,SUM($E$13:$E$22),IF($A13=Paramètres!$B$7,SUM($F$13:$F$22),0)))</f>
-        <v>1232.85600681269</v>
+        <v>1298.22324557302</v>
       </c>
       <c r="J13" s="6" t="n">
         <f aca="false">IF($A13="","",G13+D13+H13+IF(B13="Joint",E13+F13,0)-C13-I13)</f>
-        <v>1167.14399318731</v>
+        <v>1101.77675442698</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1285,11 +1305,11 @@
       </c>
       <c r="I14" s="6" t="n">
         <f aca="false">IF($A14="","",IF($A14=Paramètres!$B$6,SUM($E$13:$E$22),IF($A14=Paramètres!$B$7,SUM($F$13:$F$22),0)))</f>
-        <v>1032.14399318731</v>
+        <v>1095.77675442698</v>
       </c>
       <c r="J14" s="6" t="n">
         <f aca="false">IF($A14="","",G14+D14+H14+IF(B14="Joint",E14+F14,0)-C14-I14)</f>
-        <v>839.856006812689</v>
+        <v>776.223245573025</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1345,7 +1365,7 @@
       </c>
       <c r="C16" s="6" t="n">
         <f aca="false">IF($A16="","",SUMIFS(Charges!$F$5:$F$54,Charges!$H$5:$H$54,$A16))</f>
-        <v>1031.66666666667</v>
+        <v>1160.66666666667</v>
       </c>
       <c r="D16" s="6" t="n">
         <f aca="false">IF($A16="","",SUMIFS(Revenus!$F$5:$F$24,Revenus!$G$5:$G$24,$A16,Revenus!$B$5:$B$24,"&lt;&gt;Salaire"))</f>
@@ -1353,11 +1373,11 @@
       </c>
       <c r="E16" s="11" t="n">
         <f aca="false">IF($A16="","",IF($B16="Joint",IF($C16=0,0,($C16-$D16)*SUMIFS(Charges!$M$5:$M$54,Charges!$H$5:$H$54,$A16)/$C16),0))</f>
-        <v>428.03042541734</v>
+        <v>493.397664177676</v>
       </c>
       <c r="F16" s="11" t="n">
         <f aca="false">IF($A16="","",IF($B16="Joint",IF($C16=0,0,($C16-$D16)*SUMIFS(Charges!$N$5:$N$54,Charges!$H$5:$H$54,$A16)/$C16),0))</f>
-        <v>373.636241249327</v>
+        <v>437.269002488991</v>
       </c>
       <c r="G16" s="6" t="n">
         <f aca="false">IF($A16="","",SUMIFS(Revenus!$F$5:$F$24,Revenus!$G$5:$G$24,$A16,Revenus!$B$5:$B$24,"Salaire"))</f>
@@ -1635,7 +1655,7 @@
       <c r="B23" s="8"/>
       <c r="C23" s="9" t="n">
         <f aca="false">SUM(C13:C22)</f>
-        <v>2523</v>
+        <v>2652</v>
       </c>
       <c r="D23" s="9" t="n">
         <f aca="false">SUM(D13:D22)</f>
@@ -1643,11 +1663,11 @@
       </c>
       <c r="E23" s="9" t="n">
         <f aca="false">SUM(E13:E22)</f>
-        <v>1232.85600681269</v>
+        <v>1298.22324557302</v>
       </c>
       <c r="F23" s="9" t="n">
         <f aca="false">SUM(F13:F22)</f>
-        <v>1032.14399318731</v>
+        <v>1095.77675442698</v>
       </c>
       <c r="G23" s="9" t="n">
         <f aca="false">SUM(G13:G22)</f>
@@ -1659,11 +1679,11 @@
       </c>
       <c r="I23" s="9" t="n">
         <f aca="false">SUM(I13:I22)</f>
-        <v>2265</v>
+        <v>2394</v>
       </c>
       <c r="J23" s="9" t="n">
         <f aca="false">SUM(J13:J22)</f>
-        <v>2157</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1686,7 +1706,7 @@
       </c>
       <c r="C28" s="7" t="n">
         <f aca="false">IF($B$30=0,0,B28/$B$30)</f>
-        <v>0.626767076231999</v>
+        <v>0.596279537456008</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1695,11 +1715,11 @@
       </c>
       <c r="B29" s="6" t="n">
         <f aca="false">SUMIFS(Charges!$F$5:$F$54,Charges!$C$5:$C$54,"Variable")</f>
-        <v>941.666666666667</v>
+        <v>1070.66666666667</v>
       </c>
       <c r="C29" s="7" t="n">
         <f aca="false">IF($B$30=0,0,B29/$B$30)</f>
-        <v>0.373232923768001</v>
+        <v>0.403720462543992</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1708,7 +1728,7 @@
       </c>
       <c r="B30" s="9" t="n">
         <f aca="false">B28+B29</f>
-        <v>2523</v>
+        <v>2652</v>
       </c>
       <c r="C30" s="10" t="n">
         <f aca="false">C28+C29</f>
@@ -1731,7 +1751,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52"/>
@@ -1904,6 +1924,19 @@
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
         <v>59</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="B22" s="20" t="n">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="2" t="s">
+        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -1943,26 +1976,26 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>18</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1970,13 +2003,13 @@
         <v>41</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C5" s="13" t="s">
         <v>35</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1984,69 +2017,69 @@
         <v>44</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C6" s="13" t="s">
         <v>38</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="C8" s="13" t="s">
         <v>72</v>
       </c>
-      <c r="B8" s="13" t="s">
-        <v>69</v>
-      </c>
-      <c r="C8" s="13" t="s">
-        <v>70</v>
-      </c>
       <c r="D8" s="13" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2114,50 +2147,50 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>32</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="L4" s="4" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="M4" s="4" t="str">
         <f aca="false">"Part "&amp;Paramètres!$B$4&amp;" (€/mois)"</f>
@@ -2170,10 +2203,10 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C5" s="13" t="s">
         <v>28</v>
@@ -2189,17 +2222,17 @@
         <v>1150</v>
       </c>
       <c r="G5" s="13" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="H5" s="13" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I5" s="13"/>
       <c r="J5" s="13" t="n">
         <v>5</v>
       </c>
       <c r="K5" s="13" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="L5" s="7" t="n">
         <f aca="false">IF(A5="","",IF(K5="50/50",0.5,IF(K5="Prorata salaires",Paramètres!$B$9,IF(K5="Personne 1 seul",1,IF(K5="Personne 2 seul",0,0.5)))))</f>
@@ -2216,10 +2249,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C6" s="13" t="s">
         <v>28</v>
@@ -2235,17 +2268,17 @@
         <v>45</v>
       </c>
       <c r="G6" s="13" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="H6" s="13" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I6" s="13"/>
       <c r="J6" s="13" t="n">
         <v>5</v>
       </c>
       <c r="K6" s="13" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="L6" s="7" t="n">
         <f aca="false">IF(A6="","",IF(K6="50/50",0.5,IF(K6="Prorata salaires",Paramètres!$B$9,IF(K6="Personne 1 seul",1,IF(K6="Personne 2 seul",0,0.5)))))</f>
@@ -2262,10 +2295,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C7" s="13" t="s">
         <v>28</v>
@@ -2281,17 +2314,17 @@
         <v>108.333333333333</v>
       </c>
       <c r="G7" s="13" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="H7" s="13" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I7" s="13"/>
       <c r="J7" s="13" t="n">
         <v>15</v>
       </c>
       <c r="K7" s="13" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="L7" s="7" t="n">
         <f aca="false">IF(A7="","",IF(K7="50/50",0.5,IF(K7="Prorata salaires",Paramètres!$B$9,IF(K7="Personne 1 seul",1,IF(K7="Personne 2 seul",0,0.5)))))</f>
@@ -2308,13 +2341,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D8" s="13" t="s">
         <v>36</v>
@@ -2327,17 +2360,17 @@
         <v>130</v>
       </c>
       <c r="G8" s="13" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="H8" s="13" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I8" s="13"/>
       <c r="J8" s="13" t="n">
         <v>12</v>
       </c>
       <c r="K8" s="13" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="L8" s="7" t="n">
         <f aca="false">IF(A8="","",IF(K8="50/50",0.5,IF(K8="Prorata salaires",Paramètres!$B$9,IF(K8="Personne 1 seul",1,IF(K8="Personne 2 seul",0,0.5)))))</f>
@@ -2354,10 +2387,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C9" s="13" t="s">
         <v>28</v>
@@ -2373,17 +2406,17 @@
         <v>30</v>
       </c>
       <c r="G9" s="13" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="H9" s="13" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I9" s="13"/>
       <c r="J9" s="13" t="n">
         <v>10</v>
       </c>
       <c r="K9" s="13" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="L9" s="7" t="n">
         <f aca="false">IF(A9="","",IF(K9="50/50",0.5,IF(K9="Prorata salaires",Paramètres!$B$9,IF(K9="Personne 1 seul",1,IF(K9="Personne 2 seul",0,0.5)))))</f>
@@ -2400,10 +2433,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C10" s="13" t="s">
         <v>28</v>
@@ -2419,17 +2452,17 @@
         <v>70</v>
       </c>
       <c r="G10" s="13" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="H10" s="13" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I10" s="13"/>
       <c r="J10" s="13" t="n">
         <v>1</v>
       </c>
       <c r="K10" s="13" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="L10" s="7" t="n">
         <f aca="false">IF(A10="","",IF(K10="50/50",0.5,IF(K10="Prorata salaires",Paramètres!$B$9,IF(K10="Personne 1 seul",1,IF(K10="Personne 2 seul",0,0.5)))))</f>
@@ -2446,10 +2479,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C11" s="13" t="s">
         <v>28</v>
@@ -2465,7 +2498,7 @@
         <v>28</v>
       </c>
       <c r="G11" s="13" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="H11" s="13" t="s">
         <v>44</v>
@@ -2475,7 +2508,7 @@
         <v>8</v>
       </c>
       <c r="K11" s="13" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="L11" s="7" t="n">
         <f aca="false">IF(A11="","",IF(K11="50/50",0.5,IF(K11="Prorata salaires",Paramètres!$B$9,IF(K11="Personne 1 seul",1,IF(K11="Personne 2 seul",0,0.5)))))</f>
@@ -2492,13 +2525,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D12" s="13" t="s">
         <v>36</v>
@@ -2511,15 +2544,15 @@
         <v>600</v>
       </c>
       <c r="G12" s="13" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="H12" s="13" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I12" s="13"/>
       <c r="J12" s="13"/>
       <c r="K12" s="13" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="L12" s="7" t="n">
         <f aca="false">IF(A12="","",IF(K12="50/50",0.5,IF(K12="Prorata salaires",Paramètres!$B$9,IF(K12="Personne 1 seul",1,IF(K12="Personne 2 seul",0,0.5)))))</f>
@@ -2536,10 +2569,10 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C13" s="13" t="s">
         <v>28</v>
@@ -2555,19 +2588,19 @@
         <v>150</v>
       </c>
       <c r="G13" s="13" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="H13" s="13" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I13" s="13" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="J13" s="13" t="n">
         <v>3</v>
       </c>
       <c r="K13" s="13" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="L13" s="7" t="n">
         <f aca="false">IF(A13="","",IF(K13="50/50",0.5,IF(K13="Prorata salaires",Paramètres!$B$9,IF(K13="Personne 1 seul",1,IF(K13="Personne 2 seul",0,0.5)))))</f>
@@ -2584,13 +2617,13 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D14" s="13" t="s">
         <v>36</v>
@@ -2603,19 +2636,19 @@
         <v>90</v>
       </c>
       <c r="G14" s="13" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="H14" s="13" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I14" s="13" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="J14" s="13" t="n">
         <v>28</v>
       </c>
       <c r="K14" s="13" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="L14" s="7" t="n">
         <f aca="false">IF(A14="","",IF(K14="50/50",0.5,IF(K14="Prorata salaires",Paramètres!$B$9,IF(K14="Personne 1 seul",1,IF(K14="Personne 2 seul",0,0.5)))))</f>
@@ -2632,13 +2665,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="B15" s="13" t="s">
         <v>117</v>
       </c>
-      <c r="B15" s="13" t="s">
-        <v>115</v>
-      </c>
       <c r="C15" s="13" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D15" s="13" t="s">
         <v>45</v>
@@ -2651,15 +2684,15 @@
         <v>50</v>
       </c>
       <c r="G15" s="13" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="H15" s="13" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I15" s="13"/>
       <c r="J15" s="13"/>
       <c r="K15" s="13" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="L15" s="7" t="n">
         <f aca="false">IF(A15="","",IF(K15="50/50",0.5,IF(K15="Prorata salaires",Paramètres!$B$9,IF(K15="Personne 1 seul",1,IF(K15="Personne 2 seul",0,0.5)))))</f>
@@ -2676,13 +2709,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D16" s="13" t="s">
         <v>36</v>
@@ -2695,15 +2728,15 @@
         <v>30</v>
       </c>
       <c r="G16" s="13" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="H16" s="13" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I16" s="13"/>
       <c r="J16" s="13"/>
       <c r="K16" s="13" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="L16" s="7" t="n">
         <f aca="false">IF(A16="","",IF(K16="50/50",0.5,IF(K16="Prorata salaires",Paramètres!$B$9,IF(K16="Personne 1 seul",1,IF(K16="Personne 2 seul",0,0.5)))))</f>
@@ -2720,13 +2753,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D17" s="13" t="s">
         <v>45</v>
@@ -2739,15 +2772,15 @@
         <v>41.6666666666667</v>
       </c>
       <c r="G17" s="13" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="H17" s="13" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I17" s="13"/>
       <c r="J17" s="13"/>
       <c r="K17" s="13" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="L17" s="7" t="n">
         <f aca="false">IF(A17="","",IF(K17="50/50",0.5,IF(K17="Prorata salaires",Paramètres!$B$9,IF(K17="Personne 1 seul",1,IF(K17="Personne 2 seul",0,0.5)))))</f>
@@ -2763,31 +2796,48 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="13"/>
-      <c r="B18" s="13"/>
-      <c r="C18" s="13"/>
-      <c r="D18" s="13"/>
-      <c r="E18" s="18"/>
-      <c r="F18" s="6" t="str">
+      <c r="A18" s="13" t="s">
+        <v>124</v>
+      </c>
+      <c r="B18" s="13" t="s">
+        <v>125</v>
+      </c>
+      <c r="C18" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="D18" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="E18" s="21" t="n">
+        <f aca="false">Paramètres!$B$22*SUMIFS(Revenus!$F$5:$F$24,Revenus!$B$5:$B$24,"Salaire")</f>
+        <v>129</v>
+      </c>
+      <c r="F18" s="6" t="n">
         <f aca="false">IF(A18="","",IFERROR(E18/INDEX(Paramètres!$E$4:$E$7,MATCH(D18,Paramètres!$D$4:$D$7,0)),0))</f>
-        <v/>
-      </c>
-      <c r="G18" s="13"/>
-      <c r="H18" s="13"/>
+        <v>129</v>
+      </c>
+      <c r="G18" s="13" t="s">
+        <v>113</v>
+      </c>
+      <c r="H18" s="13" t="s">
+        <v>74</v>
+      </c>
       <c r="I18" s="13"/>
       <c r="J18" s="13"/>
-      <c r="K18" s="13"/>
-      <c r="L18" s="7" t="str">
+      <c r="K18" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="L18" s="7" t="n">
         <f aca="false">IF(A18="","",IF(K18="50/50",0.5,IF(K18="Prorata salaires",Paramètres!$B$9,IF(K18="Personne 1 seul",1,IF(K18="Personne 2 seul",0,0.5)))))</f>
-        <v/>
-      </c>
-      <c r="M18" s="6" t="str">
+        <v>0.5</v>
+      </c>
+      <c r="M18" s="6" t="n">
         <f aca="false">IF(A18="","",F18*L18)</f>
-        <v/>
-      </c>
-      <c r="N18" s="6" t="str">
+        <v>64.5</v>
+      </c>
+      <c r="N18" s="6" t="n">
         <f aca="false">IF(A18="","",F18-M18)</f>
-        <v/>
+        <v>64.5</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3799,20 +3849,20 @@
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="20" t="s">
-        <v>122</v>
+      <c r="A55" s="22" t="s">
+        <v>126</v>
       </c>
       <c r="F55" s="9" t="n">
         <f aca="false">SUM(F5:F54)</f>
-        <v>2523</v>
+        <v>2652</v>
       </c>
       <c r="M55" s="9" t="n">
         <f aca="false">SUM(M5:M54)</f>
-        <v>1355.65891472868</v>
+        <v>1420.15891472868</v>
       </c>
       <c r="N55" s="9" t="n">
         <f aca="false">SUM(N5:N54)</f>
-        <v>1167.34108527132</v>
+        <v>1231.84108527132</v>
       </c>
     </row>
   </sheetData>
@@ -3867,17 +3917,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>18</v>
@@ -3886,27 +3936,27 @@
         <v>3</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>32</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="C5" s="13" t="s">
         <v>35</v>
@@ -3930,10 +3980,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="C6" s="13" t="s">
         <v>38</v>
@@ -3957,13 +4007,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="D7" s="18" t="n">
         <v>140</v>
@@ -3976,7 +4026,7 @@
         <v>140</v>
       </c>
       <c r="G7" s="13" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="H7" s="13" t="n">
         <v>5</v>
@@ -3984,13 +4034,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="D8" s="18" t="n">
         <v>270</v>
@@ -4003,7 +4053,7 @@
         <v>90</v>
       </c>
       <c r="G8" s="13" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="H8" s="13" t="n">
         <v>5</v>
@@ -4218,8 +4268,8 @@
       <c r="H24" s="13"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="20" t="s">
-        <v>122</v>
+      <c r="A25" s="22" t="s">
+        <v>126</v>
       </c>
       <c r="F25" s="9" t="n">
         <f aca="false">SUM(F5:F24)</f>
@@ -4267,43 +4317,43 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>3</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>32</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="B5" s="13" t="s">
         <v>35</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D5" s="13" t="s">
         <v>36</v>
@@ -4318,13 +4368,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B6" s="13" t="s">
         <v>35</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="D6" s="13" t="s">
         <v>39</v>
@@ -4339,13 +4389,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="B7" s="13" t="s">
         <v>35</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D7" s="13" t="s">
         <v>36</v>
@@ -4766,8 +4816,8 @@
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="20" t="s">
-        <v>122</v>
+      <c r="A45" s="22" t="s">
+        <v>126</v>
       </c>
       <c r="F45" s="9" t="n">
         <f aca="false">SUM(F5:F44)</f>
@@ -4776,12 +4826,12 @@
     </row>
   </sheetData>
   <dataValidations count="2">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B5:B44" type="list">
+      <formula1>Paramètres!$B$4:$B$5</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D5:D44" type="list">
       <formula1>"Mensuelle,Trimestrielle,Semestrielle,Annuelle"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B5:B44" type="list">
-      <formula1>Paramètres!$B$4:$B$5</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Ajout du suivi des imprévus et du livret imprévus
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KqkJNWVZSWN9upSPoUaH5h
</commit_message>
<xml_diff>
--- a/suivi_comptes.xlsx
+++ b/suivi_comptes.xlsx
@@ -14,6 +14,7 @@
     <sheet name="Charges" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Revenus" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="Charges perso" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Imprévus" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="160">
   <si>
     <t xml:space="preserve">Synthèse mensuelle</t>
   </si>
@@ -270,6 +271,12 @@
     <t xml:space="preserve">Épargne (reçoit des virements)</t>
   </si>
   <si>
+    <t xml:space="preserve">Livret imprévus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Provision pour les dépenses imprévues</t>
+  </si>
+  <si>
     <t xml:space="preserve">Charges (dépenses récurrentes)</t>
   </si>
   <si>
@@ -454,17 +461,64 @@
   </si>
   <si>
     <t xml:space="preserve">Abonnement musique</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Suivi des imprévus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Notez chaque dépense imprévue ici (date, libellé, montant). Le solde de la provision se met à jour tout seul.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Provision mensuelle (ligne « Imprévus » de Charges)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Début du suivi (1er du mois)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Solde de départ du livret imprévus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mois provisionnés (mois en cours inclus)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total provisionné</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total dépensé en imprévus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Solde de la provision</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Solde négatif = la provision n'a pas suffi : à combler avec l'épargne ou le reste libre.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Montant (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Payé depuis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pare-brise</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dentiste</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0.00&quot; €&quot;;\-#,##0.00&quot; €&quot;;\-"/>
     <numFmt numFmtId="166" formatCode="0%"/>
     <numFmt numFmtId="167" formatCode="0.0%"/>
+    <numFmt numFmtId="168" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="169" formatCode="0"/>
   </numFmts>
   <fonts count="14">
     <font>
@@ -639,7 +693,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="26">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -729,6 +783,18 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1483,43 +1549,43 @@
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="str">
         <f aca="false">IF(Comptes!A11="","",Comptes!A11)</f>
-        <v/>
+        <v>Livret imprévus</v>
       </c>
       <c r="B19" s="5" t="str">
         <f aca="false">IF($A19="","",Comptes!B11)</f>
-        <v/>
-      </c>
-      <c r="C19" s="6" t="str">
+        <v>Épargne</v>
+      </c>
+      <c r="C19" s="6" t="n">
         <f aca="false">IF($A19="","",SUMIFS(Charges!$F$5:$F$54,Charges!$H$5:$H$54,$A19))</f>
-        <v/>
-      </c>
-      <c r="D19" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="D19" s="6" t="n">
         <f aca="false">IF($A19="","",SUMIFS(Revenus!$F$5:$F$24,Revenus!$G$5:$G$24,$A19,Revenus!$B$5:$B$24,"&lt;&gt;Salaire"))</f>
-        <v/>
-      </c>
-      <c r="E19" s="11" t="str">
+        <v>0</v>
+      </c>
+      <c r="E19" s="11" t="n">
         <f aca="false">IF($A19="","",IF($B19="Joint",IF($C19=0,0,($C19-$D19)*SUMIFS(Charges!$M$5:$M$54,Charges!$H$5:$H$54,$A19)/$C19),0))</f>
-        <v/>
-      </c>
-      <c r="F19" s="11" t="str">
+        <v>0</v>
+      </c>
+      <c r="F19" s="11" t="n">
         <f aca="false">IF($A19="","",IF($B19="Joint",IF($C19=0,0,($C19-$D19)*SUMIFS(Charges!$N$5:$N$54,Charges!$H$5:$H$54,$A19)/$C19),0))</f>
-        <v/>
-      </c>
-      <c r="G19" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="G19" s="6" t="n">
         <f aca="false">IF($A19="","",SUMIFS(Revenus!$F$5:$F$24,Revenus!$G$5:$G$24,$A19,Revenus!$B$5:$B$24,"Salaire"))</f>
-        <v/>
-      </c>
-      <c r="H19" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="H19" s="6" t="n">
         <f aca="false">IF($A19="","",SUMIFS(Charges!$F$5:$F$54,Charges!$I$5:$I$54,$A19,Charges!$G$5:$G$54,"Virement"))</f>
-        <v/>
-      </c>
-      <c r="I19" s="6" t="str">
+        <v>129</v>
+      </c>
+      <c r="I19" s="6" t="n">
         <f aca="false">IF($A19="","",IF($A19=Paramètres!$B$6,SUM($E$13:$E$22),IF($A19=Paramètres!$B$7,SUM($F$13:$F$22),0)))</f>
-        <v/>
-      </c>
-      <c r="J19" s="6" t="str">
+        <v>0</v>
+      </c>
+      <c r="J19" s="6" t="n">
         <f aca="false">IF($A19="","",G19+D19+H19+IF(B19="Joint",E19+F19,0)-C19-I19)</f>
-        <v/>
+        <v>129</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1675,7 +1741,7 @@
       </c>
       <c r="H23" s="9" t="n">
         <f aca="false">SUM(H13:H22)</f>
-        <v>150</v>
+        <v>279</v>
       </c>
       <c r="I23" s="9" t="n">
         <f aca="false">SUM(I13:I22)</f>
@@ -1683,7 +1749,7 @@
       </c>
       <c r="J23" s="9" t="n">
         <f aca="false">SUM(J13:J22)</f>
-        <v>2028</v>
+        <v>2157</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2083,10 +2149,18 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="13"/>
-      <c r="B11" s="13"/>
-      <c r="C11" s="13"/>
-      <c r="D11" s="13"/>
+      <c r="A11" s="13" t="s">
+        <v>81</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="C11" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="D11" s="13" t="s">
+        <v>82</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13"/>
@@ -2147,50 +2221,50 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>32</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="L4" s="4" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="M4" s="4" t="str">
         <f aca="false">"Part "&amp;Paramètres!$B$4&amp;" (€/mois)"</f>
@@ -2203,10 +2277,10 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C5" s="13" t="s">
         <v>28</v>
@@ -2222,7 +2296,7 @@
         <v>1150</v>
       </c>
       <c r="G5" s="13" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="H5" s="13" t="s">
         <v>70</v>
@@ -2232,7 +2306,7 @@
         <v>5</v>
       </c>
       <c r="K5" s="13" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="L5" s="7" t="n">
         <f aca="false">IF(A5="","",IF(K5="50/50",0.5,IF(K5="Prorata salaires",Paramètres!$B$9,IF(K5="Personne 1 seul",1,IF(K5="Personne 2 seul",0,0.5)))))</f>
@@ -2249,10 +2323,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C6" s="13" t="s">
         <v>28</v>
@@ -2268,7 +2342,7 @@
         <v>45</v>
       </c>
       <c r="G6" s="13" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="H6" s="13" t="s">
         <v>70</v>
@@ -2278,7 +2352,7 @@
         <v>5</v>
       </c>
       <c r="K6" s="13" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="L6" s="7" t="n">
         <f aca="false">IF(A6="","",IF(K6="50/50",0.5,IF(K6="Prorata salaires",Paramètres!$B$9,IF(K6="Personne 1 seul",1,IF(K6="Personne 2 seul",0,0.5)))))</f>
@@ -2295,10 +2369,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C7" s="13" t="s">
         <v>28</v>
@@ -2314,7 +2388,7 @@
         <v>108.333333333333</v>
       </c>
       <c r="G7" s="13" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="H7" s="13" t="s">
         <v>70</v>
@@ -2324,7 +2398,7 @@
         <v>15</v>
       </c>
       <c r="K7" s="13" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="L7" s="7" t="n">
         <f aca="false">IF(A7="","",IF(K7="50/50",0.5,IF(K7="Prorata salaires",Paramètres!$B$9,IF(K7="Personne 1 seul",1,IF(K7="Personne 2 seul",0,0.5)))))</f>
@@ -2341,13 +2415,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D8" s="13" t="s">
         <v>36</v>
@@ -2360,7 +2434,7 @@
         <v>130</v>
       </c>
       <c r="G8" s="13" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="H8" s="13" t="s">
         <v>70</v>
@@ -2370,7 +2444,7 @@
         <v>12</v>
       </c>
       <c r="K8" s="13" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="L8" s="7" t="n">
         <f aca="false">IF(A8="","",IF(K8="50/50",0.5,IF(K8="Prorata salaires",Paramètres!$B$9,IF(K8="Personne 1 seul",1,IF(K8="Personne 2 seul",0,0.5)))))</f>
@@ -2387,10 +2461,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C9" s="13" t="s">
         <v>28</v>
@@ -2406,7 +2480,7 @@
         <v>30</v>
       </c>
       <c r="G9" s="13" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="H9" s="13" t="s">
         <v>76</v>
@@ -2416,7 +2490,7 @@
         <v>10</v>
       </c>
       <c r="K9" s="13" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="L9" s="7" t="n">
         <f aca="false">IF(A9="","",IF(K9="50/50",0.5,IF(K9="Prorata salaires",Paramètres!$B$9,IF(K9="Personne 1 seul",1,IF(K9="Personne 2 seul",0,0.5)))))</f>
@@ -2433,10 +2507,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C10" s="13" t="s">
         <v>28</v>
@@ -2452,7 +2526,7 @@
         <v>70</v>
       </c>
       <c r="G10" s="13" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="H10" s="13" t="s">
         <v>74</v>
@@ -2462,7 +2536,7 @@
         <v>1</v>
       </c>
       <c r="K10" s="13" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="L10" s="7" t="n">
         <f aca="false">IF(A10="","",IF(K10="50/50",0.5,IF(K10="Prorata salaires",Paramètres!$B$9,IF(K10="Personne 1 seul",1,IF(K10="Personne 2 seul",0,0.5)))))</f>
@@ -2479,10 +2553,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C11" s="13" t="s">
         <v>28</v>
@@ -2498,7 +2572,7 @@
         <v>28</v>
       </c>
       <c r="G11" s="13" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="H11" s="13" t="s">
         <v>44</v>
@@ -2508,7 +2582,7 @@
         <v>8</v>
       </c>
       <c r="K11" s="13" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L11" s="7" t="n">
         <f aca="false">IF(A11="","",IF(K11="50/50",0.5,IF(K11="Prorata salaires",Paramètres!$B$9,IF(K11="Personne 1 seul",1,IF(K11="Personne 2 seul",0,0.5)))))</f>
@@ -2525,13 +2599,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D12" s="13" t="s">
         <v>36</v>
@@ -2544,7 +2618,7 @@
         <v>600</v>
       </c>
       <c r="G12" s="13" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="H12" s="13" t="s">
         <v>74</v>
@@ -2552,7 +2626,7 @@
       <c r="I12" s="13"/>
       <c r="J12" s="13"/>
       <c r="K12" s="13" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="L12" s="7" t="n">
         <f aca="false">IF(A12="","",IF(K12="50/50",0.5,IF(K12="Prorata salaires",Paramètres!$B$9,IF(K12="Personne 1 seul",1,IF(K12="Personne 2 seul",0,0.5)))))</f>
@@ -2569,7 +2643,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B13" s="13" t="s">
         <v>79</v>
@@ -2588,7 +2662,7 @@
         <v>150</v>
       </c>
       <c r="G13" s="13" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="H13" s="13" t="s">
         <v>74</v>
@@ -2600,7 +2674,7 @@
         <v>3</v>
       </c>
       <c r="K13" s="13" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="L13" s="7" t="n">
         <f aca="false">IF(A13="","",IF(K13="50/50",0.5,IF(K13="Prorata salaires",Paramètres!$B$9,IF(K13="Personne 1 seul",1,IF(K13="Personne 2 seul",0,0.5)))))</f>
@@ -2617,13 +2691,13 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D14" s="13" t="s">
         <v>36</v>
@@ -2636,19 +2710,19 @@
         <v>90</v>
       </c>
       <c r="G14" s="13" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="H14" s="13" t="s">
         <v>74</v>
       </c>
       <c r="I14" s="13" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="J14" s="13" t="n">
         <v>28</v>
       </c>
       <c r="K14" s="13" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="L14" s="7" t="n">
         <f aca="false">IF(A14="","",IF(K14="50/50",0.5,IF(K14="Prorata salaires",Paramètres!$B$9,IF(K14="Personne 1 seul",1,IF(K14="Personne 2 seul",0,0.5)))))</f>
@@ -2665,13 +2739,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
+        <v>121</v>
+      </c>
+      <c r="B15" s="13" t="s">
         <v>119</v>
       </c>
-      <c r="B15" s="13" t="s">
-        <v>117</v>
-      </c>
       <c r="C15" s="13" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D15" s="13" t="s">
         <v>45</v>
@@ -2684,7 +2758,7 @@
         <v>50</v>
       </c>
       <c r="G15" s="13" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="H15" s="13" t="s">
         <v>74</v>
@@ -2692,7 +2766,7 @@
       <c r="I15" s="13"/>
       <c r="J15" s="13"/>
       <c r="K15" s="13" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="L15" s="7" t="n">
         <f aca="false">IF(A15="","",IF(K15="50/50",0.5,IF(K15="Prorata salaires",Paramètres!$B$9,IF(K15="Personne 1 seul",1,IF(K15="Personne 2 seul",0,0.5)))))</f>
@@ -2709,13 +2783,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D16" s="13" t="s">
         <v>36</v>
@@ -2728,7 +2802,7 @@
         <v>30</v>
       </c>
       <c r="G16" s="13" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="H16" s="13" t="s">
         <v>74</v>
@@ -2736,7 +2810,7 @@
       <c r="I16" s="13"/>
       <c r="J16" s="13"/>
       <c r="K16" s="13" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="L16" s="7" t="n">
         <f aca="false">IF(A16="","",IF(K16="50/50",0.5,IF(K16="Prorata salaires",Paramètres!$B$9,IF(K16="Personne 1 seul",1,IF(K16="Personne 2 seul",0,0.5)))))</f>
@@ -2753,13 +2827,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D17" s="13" t="s">
         <v>45</v>
@@ -2772,7 +2846,7 @@
         <v>41.6666666666667</v>
       </c>
       <c r="G17" s="13" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="H17" s="13" t="s">
         <v>74</v>
@@ -2780,7 +2854,7 @@
       <c r="I17" s="13"/>
       <c r="J17" s="13"/>
       <c r="K17" s="13" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="L17" s="7" t="n">
         <f aca="false">IF(A17="","",IF(K17="50/50",0.5,IF(K17="Prorata salaires",Paramètres!$B$9,IF(K17="Personne 1 seul",1,IF(K17="Personne 2 seul",0,0.5)))))</f>
@@ -2797,13 +2871,13 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D18" s="13" t="s">
         <v>36</v>
@@ -2817,15 +2891,19 @@
         <v>129</v>
       </c>
       <c r="G18" s="13" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="H18" s="13" t="s">
         <v>74</v>
       </c>
-      <c r="I18" s="13"/>
-      <c r="J18" s="13"/>
+      <c r="I18" s="13" t="s">
+        <v>81</v>
+      </c>
+      <c r="J18" s="13" t="n">
+        <v>3</v>
+      </c>
       <c r="K18" s="13" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="L18" s="7" t="n">
         <f aca="false">IF(A18="","",IF(K18="50/50",0.5,IF(K18="Prorata salaires",Paramètres!$B$9,IF(K18="Personne 1 seul",1,IF(K18="Personne 2 seul",0,0.5)))))</f>
@@ -3850,7 +3928,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="22" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="F55" s="9" t="n">
         <f aca="false">SUM(F5:F54)</f>
@@ -3917,17 +3995,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>18</v>
@@ -3936,27 +4014,27 @@
         <v>3</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>32</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C5" s="13" t="s">
         <v>35</v>
@@ -3980,10 +4058,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C6" s="13" t="s">
         <v>38</v>
@@ -4007,13 +4085,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D7" s="18" t="n">
         <v>140</v>
@@ -4034,13 +4112,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
+        <v>138</v>
+      </c>
+      <c r="B8" s="13" t="s">
         <v>136</v>
       </c>
-      <c r="B8" s="13" t="s">
-        <v>134</v>
-      </c>
       <c r="C8" s="13" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D8" s="18" t="n">
         <v>270</v>
@@ -4269,7 +4347,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="22" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="F25" s="9" t="n">
         <f aca="false">SUM(F5:F24)</f>
@@ -4317,43 +4395,43 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>3</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>32</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B5" s="13" t="s">
         <v>35</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="D5" s="13" t="s">
         <v>36</v>
@@ -4368,13 +4446,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B6" s="13" t="s">
         <v>35</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D6" s="13" t="s">
         <v>39</v>
@@ -4389,13 +4467,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B7" s="13" t="s">
         <v>35</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D7" s="13" t="s">
         <v>36</v>
@@ -4817,7 +4895,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="22" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="F45" s="9" t="n">
         <f aca="false">SUM(F5:F44)</f>
@@ -4843,4 +4921,441 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D62"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="22"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="23" t="s">
+        <v>147</v>
+      </c>
+      <c r="B4" s="6" t="n">
+        <f aca="false">SUMIFS(Charges!$F$5:$F$54,Charges!$B$5:$B$54,"Imprévus")</f>
+        <v>129</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="B5" s="24" t="n">
+        <v>46266</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="23" t="s">
+        <v>149</v>
+      </c>
+      <c r="B6" s="18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="23" t="s">
+        <v>150</v>
+      </c>
+      <c r="B7" s="25" t="n">
+        <f aca="true">MAX(0,(YEAR(TODAY())-YEAR(B5))*12+MONTH(TODAY())-MONTH(B5)+1)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="23" t="s">
+        <v>151</v>
+      </c>
+      <c r="B8" s="6" t="n">
+        <f aca="false">B6+B4*B7</f>
+        <v>258</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="23" t="s">
+        <v>152</v>
+      </c>
+      <c r="B9" s="6" t="n">
+        <f aca="false">SUM(C13:C62)</f>
+        <v>305</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="B10" s="9" t="n">
+        <f aca="false">B8-B9</f>
+        <v>-47</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="2" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="24" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>158</v>
+      </c>
+      <c r="C13" s="18" t="n">
+        <v>220</v>
+      </c>
+      <c r="D13" s="13" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="24" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B14" s="13" t="s">
+        <v>159</v>
+      </c>
+      <c r="C14" s="18" t="n">
+        <v>85</v>
+      </c>
+      <c r="D14" s="13" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="24"/>
+      <c r="B15" s="13"/>
+      <c r="C15" s="18"/>
+      <c r="D15" s="13"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="24"/>
+      <c r="B16" s="13"/>
+      <c r="C16" s="18"/>
+      <c r="D16" s="13"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="24"/>
+      <c r="B17" s="13"/>
+      <c r="C17" s="18"/>
+      <c r="D17" s="13"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="24"/>
+      <c r="B18" s="13"/>
+      <c r="C18" s="18"/>
+      <c r="D18" s="13"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="24"/>
+      <c r="B19" s="13"/>
+      <c r="C19" s="18"/>
+      <c r="D19" s="13"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="24"/>
+      <c r="B20" s="13"/>
+      <c r="C20" s="18"/>
+      <c r="D20" s="13"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="24"/>
+      <c r="B21" s="13"/>
+      <c r="C21" s="18"/>
+      <c r="D21" s="13"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="24"/>
+      <c r="B22" s="13"/>
+      <c r="C22" s="18"/>
+      <c r="D22" s="13"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="24"/>
+      <c r="B23" s="13"/>
+      <c r="C23" s="18"/>
+      <c r="D23" s="13"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="24"/>
+      <c r="B24" s="13"/>
+      <c r="C24" s="18"/>
+      <c r="D24" s="13"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="24"/>
+      <c r="B25" s="13"/>
+      <c r="C25" s="18"/>
+      <c r="D25" s="13"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="24"/>
+      <c r="B26" s="13"/>
+      <c r="C26" s="18"/>
+      <c r="D26" s="13"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="24"/>
+      <c r="B27" s="13"/>
+      <c r="C27" s="18"/>
+      <c r="D27" s="13"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="24"/>
+      <c r="B28" s="13"/>
+      <c r="C28" s="18"/>
+      <c r="D28" s="13"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="24"/>
+      <c r="B29" s="13"/>
+      <c r="C29" s="18"/>
+      <c r="D29" s="13"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="24"/>
+      <c r="B30" s="13"/>
+      <c r="C30" s="18"/>
+      <c r="D30" s="13"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="24"/>
+      <c r="B31" s="13"/>
+      <c r="C31" s="18"/>
+      <c r="D31" s="13"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="24"/>
+      <c r="B32" s="13"/>
+      <c r="C32" s="18"/>
+      <c r="D32" s="13"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="24"/>
+      <c r="B33" s="13"/>
+      <c r="C33" s="18"/>
+      <c r="D33" s="13"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="24"/>
+      <c r="B34" s="13"/>
+      <c r="C34" s="18"/>
+      <c r="D34" s="13"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="24"/>
+      <c r="B35" s="13"/>
+      <c r="C35" s="18"/>
+      <c r="D35" s="13"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="24"/>
+      <c r="B36" s="13"/>
+      <c r="C36" s="18"/>
+      <c r="D36" s="13"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="24"/>
+      <c r="B37" s="13"/>
+      <c r="C37" s="18"/>
+      <c r="D37" s="13"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="24"/>
+      <c r="B38" s="13"/>
+      <c r="C38" s="18"/>
+      <c r="D38" s="13"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="24"/>
+      <c r="B39" s="13"/>
+      <c r="C39" s="18"/>
+      <c r="D39" s="13"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="24"/>
+      <c r="B40" s="13"/>
+      <c r="C40" s="18"/>
+      <c r="D40" s="13"/>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="24"/>
+      <c r="B41" s="13"/>
+      <c r="C41" s="18"/>
+      <c r="D41" s="13"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="24"/>
+      <c r="B42" s="13"/>
+      <c r="C42" s="18"/>
+      <c r="D42" s="13"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="24"/>
+      <c r="B43" s="13"/>
+      <c r="C43" s="18"/>
+      <c r="D43" s="13"/>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="24"/>
+      <c r="B44" s="13"/>
+      <c r="C44" s="18"/>
+      <c r="D44" s="13"/>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="24"/>
+      <c r="B45" s="13"/>
+      <c r="C45" s="18"/>
+      <c r="D45" s="13"/>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="24"/>
+      <c r="B46" s="13"/>
+      <c r="C46" s="18"/>
+      <c r="D46" s="13"/>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="24"/>
+      <c r="B47" s="13"/>
+      <c r="C47" s="18"/>
+      <c r="D47" s="13"/>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="24"/>
+      <c r="B48" s="13"/>
+      <c r="C48" s="18"/>
+      <c r="D48" s="13"/>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="24"/>
+      <c r="B49" s="13"/>
+      <c r="C49" s="18"/>
+      <c r="D49" s="13"/>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="24"/>
+      <c r="B50" s="13"/>
+      <c r="C50" s="18"/>
+      <c r="D50" s="13"/>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="24"/>
+      <c r="B51" s="13"/>
+      <c r="C51" s="18"/>
+      <c r="D51" s="13"/>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="24"/>
+      <c r="B52" s="13"/>
+      <c r="C52" s="18"/>
+      <c r="D52" s="13"/>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="24"/>
+      <c r="B53" s="13"/>
+      <c r="C53" s="18"/>
+      <c r="D53" s="13"/>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="24"/>
+      <c r="B54" s="13"/>
+      <c r="C54" s="18"/>
+      <c r="D54" s="13"/>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="24"/>
+      <c r="B55" s="13"/>
+      <c r="C55" s="18"/>
+      <c r="D55" s="13"/>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="24"/>
+      <c r="B56" s="13"/>
+      <c r="C56" s="18"/>
+      <c r="D56" s="13"/>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="24"/>
+      <c r="B57" s="13"/>
+      <c r="C57" s="18"/>
+      <c r="D57" s="13"/>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="24"/>
+      <c r="B58" s="13"/>
+      <c r="C58" s="18"/>
+      <c r="D58" s="13"/>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="24"/>
+      <c r="B59" s="13"/>
+      <c r="C59" s="18"/>
+      <c r="D59" s="13"/>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="24"/>
+      <c r="B60" s="13"/>
+      <c r="C60" s="18"/>
+      <c r="D60" s="13"/>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="24"/>
+      <c r="B61" s="13"/>
+      <c r="C61" s="18"/>
+      <c r="D61" s="13"/>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="24"/>
+      <c r="B62" s="13"/>
+      <c r="C62" s="18"/>
+      <c r="D62" s="13"/>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D13:D62" type="list">
+      <formula1>Comptes!$A$5:$A$14</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Ajout des modes de paiement chèque et espèces
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KqkJNWVZSWN9upSPoUaH5h
</commit_message>
<xml_diff>
--- a/suivi_comptes.xlsx
+++ b/suivi_comptes.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="161">
   <si>
     <t xml:space="preserve">Synthèse mensuelle</t>
   </si>
@@ -398,6 +398,9 @@
   </si>
   <si>
     <t xml:space="preserve">Santé</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chèque</t>
   </si>
   <si>
     <t xml:space="preserve">Cadeaux &amp; fêtes (enveloppe lissée)</t>
@@ -2802,7 +2805,7 @@
         <v>30</v>
       </c>
       <c r="G16" s="13" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="H16" s="13" t="s">
         <v>74</v>
@@ -2827,10 +2830,10 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C17" s="13" t="s">
         <v>105</v>
@@ -2871,10 +2874,10 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C18" s="13" t="s">
         <v>105</v>
@@ -3928,7 +3931,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="22" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F55" s="9" t="n">
         <f aca="false">SUM(F5:F54)</f>
@@ -3954,7 +3957,7 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G5:G54" type="list">
-      <formula1>"Prélèvement,Virement,Carte"</formula1>
+      <formula1>"Prélèvement,Virement,Carte,Chèque,Espèces"</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H5:H54" type="list">
@@ -3995,12 +3998,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4023,7 +4026,7 @@
         <v>89</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H4" s="4" t="s">
         <v>93</v>
@@ -4031,10 +4034,10 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C5" s="13" t="s">
         <v>35</v>
@@ -4058,10 +4061,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
+        <v>135</v>
+      </c>
+      <c r="B6" s="13" t="s">
         <v>134</v>
-      </c>
-      <c r="B6" s="13" t="s">
-        <v>133</v>
       </c>
       <c r="C6" s="13" t="s">
         <v>38</v>
@@ -4085,13 +4088,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D7" s="18" t="n">
         <v>140</v>
@@ -4112,13 +4115,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
+        <v>139</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>137</v>
+      </c>
+      <c r="C8" s="13" t="s">
         <v>138</v>
-      </c>
-      <c r="B8" s="13" t="s">
-        <v>136</v>
-      </c>
-      <c r="C8" s="13" t="s">
-        <v>137</v>
       </c>
       <c r="D8" s="18" t="n">
         <v>270</v>
@@ -4347,7 +4350,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="22" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F25" s="9" t="n">
         <f aca="false">SUM(F5:F24)</f>
@@ -4395,12 +4398,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4425,13 +4428,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B5" s="13" t="s">
         <v>35</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D5" s="13" t="s">
         <v>36</v>
@@ -4446,13 +4449,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B6" s="13" t="s">
         <v>35</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D6" s="13" t="s">
         <v>39</v>
@@ -4467,7 +4470,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B7" s="13" t="s">
         <v>35</v>
@@ -4895,7 +4898,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="22" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F45" s="9" t="n">
         <f aca="false">SUM(F5:F44)</f>
@@ -4904,12 +4907,12 @@
     </row>
   </sheetData>
   <dataValidations count="2">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D5:D44" type="list">
+      <formula1>"Mensuelle,Trimestrielle,Semestrielle,Annuelle"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B5:B44" type="list">
       <formula1>Paramètres!$B$4:$B$5</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D5:D44" type="list">
-      <formula1>"Mensuelle,Trimestrielle,Semestrielle,Annuelle"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -4939,17 +4942,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="23" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B4" s="6" t="n">
         <f aca="false">SUMIFS(Charges!$F$5:$F$54,Charges!$B$5:$B$54,"Imprévus")</f>
@@ -4958,7 +4961,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="23" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B5" s="24" t="n">
         <v>46266</v>
@@ -4966,7 +4969,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="23" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B6" s="18" t="n">
         <v>0</v>
@@ -4974,7 +4977,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="23" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B7" s="25" t="n">
         <f aca="true">MAX(0,(YEAR(TODAY())-YEAR(B5))*12+MONTH(TODAY())-MONTH(B5)+1)</f>
@@ -4983,7 +4986,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="23" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B8" s="6" t="n">
         <f aca="false">B6+B4*B7</f>
@@ -4992,7 +4995,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="23" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B9" s="6" t="n">
         <f aca="false">SUM(C13:C62)</f>
@@ -5001,7 +5004,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B10" s="9" t="n">
         <f aca="false">B8-B9</f>
@@ -5010,21 +5013,21 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>85</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5032,7 +5035,7 @@
         <v>46285</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C13" s="18" t="n">
         <v>220</v>
@@ -5046,7 +5049,7 @@
         <v>46300</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C14" s="18" t="n">
         <v>85</v>

</xml_diff>

<commit_message>
Ajout d'exemples de retraits d'espèces depuis le compte joint
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KqkJNWVZSWN9upSPoUaH5h
</commit_message>
<xml_diff>
--- a/suivi_comptes.xlsx
+++ b/suivi_comptes.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="166">
   <si>
     <t xml:space="preserve">Synthèse mensuelle</t>
   </si>
@@ -413,6 +413,21 @@
   </si>
   <si>
     <t xml:space="preserve">Imprévus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aide à domicile (retrait espèces)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Services</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Espèces</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Argent de poche enfants (retrait espèces)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marché &amp; petits commerces (retrait espèces)</t>
   </si>
   <si>
     <t xml:space="preserve">TOTAL mensuel</t>
@@ -1127,7 +1142,7 @@
       </c>
       <c r="C5" s="6" t="n">
         <f aca="false">SUM(E$13:E$22)</f>
-        <v>1298.22324557302</v>
+        <v>1404.28586025397</v>
       </c>
       <c r="D5" s="6" t="n">
         <f aca="false">IFERROR(INDEX($C$13:$C$22,MATCH(Paramètres!$B$6,$A$13:$A$22,0)),0)</f>
@@ -1135,15 +1150,15 @@
       </c>
       <c r="E5" s="6" t="n">
         <f aca="false">C5+D5</f>
-        <v>1298.22324557302</v>
+        <v>1404.28586025397</v>
       </c>
       <c r="F5" s="7" t="n">
         <f aca="false">IF(B5=0,0,E5/B5)</f>
-        <v>0.540926352322094</v>
+        <v>0.585119108439156</v>
       </c>
       <c r="G5" s="6" t="n">
         <f aca="false">IFERROR(INDEX($J$13:$J$22,MATCH(Paramètres!$B$6,$A$13:$A$22,0)),0)</f>
-        <v>1101.77675442698</v>
+        <v>995.714139746026</v>
       </c>
       <c r="H5" s="6" t="n">
         <f aca="false">IF(Paramètres!B$15="Forfait",Paramètres!B$16,SUMIFS('Charges perso'!$F$5:$F$44,'Charges perso'!$B$5:$B$44,A5))</f>
@@ -1151,15 +1166,15 @@
       </c>
       <c r="I5" s="6" t="n">
         <f aca="false">G5-H5</f>
-        <v>1015.77675442698</v>
+        <v>909.714139746026</v>
       </c>
       <c r="J5" s="6" t="n">
         <f aca="false">MAX(0,IF(Paramètres!B$17="Pourcentage",Paramètres!B$18*MAX(0,I5),Paramètres!B$19))</f>
-        <v>304.733026328093</v>
+        <v>272.914241923808</v>
       </c>
       <c r="K5" s="6" t="n">
         <f aca="false">I5-J5</f>
-        <v>711.043728098883</v>
+        <v>636.799897822218</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1173,7 +1188,7 @@
       </c>
       <c r="C6" s="6" t="n">
         <f aca="false">SUM(F$13:F$22)</f>
-        <v>1095.77675442698</v>
+        <v>1199.71413974603</v>
       </c>
       <c r="D6" s="6" t="n">
         <f aca="false">IFERROR(INDEX($C$13:$C$22,MATCH(Paramètres!$B$7,$A$13:$A$22,0)),0)</f>
@@ -1181,15 +1196,15 @@
       </c>
       <c r="E6" s="6" t="n">
         <f aca="false">C6+D6</f>
-        <v>1123.77675442698</v>
+        <v>1227.71413974603</v>
       </c>
       <c r="F6" s="7" t="n">
         <f aca="false">IF(B6=0,0,E6/B6)</f>
-        <v>0.591461449698408</v>
+        <v>0.646165336708435</v>
       </c>
       <c r="G6" s="6" t="n">
         <f aca="false">IFERROR(INDEX($J$13:$J$22,MATCH(Paramètres!$B$7,$A$13:$A$22,0)),0)</f>
-        <v>776.223245573025</v>
+        <v>672.285860253974</v>
       </c>
       <c r="H6" s="6" t="n">
         <f aca="false">IF(Paramètres!C$15="Forfait",Paramètres!C$16,SUMIFS('Charges perso'!$F$5:$F$44,'Charges perso'!$B$5:$B$44,A6))</f>
@@ -1197,7 +1212,7 @@
       </c>
       <c r="I6" s="6" t="n">
         <f aca="false">G6-H6</f>
-        <v>426.223245573025</v>
+        <v>322.285860253974</v>
       </c>
       <c r="J6" s="6" t="n">
         <f aca="false">MAX(0,IF(Paramètres!C$17="Pourcentage",Paramètres!C$18*MAX(0,I6),Paramètres!C$19))</f>
@@ -1205,7 +1220,7 @@
       </c>
       <c r="K6" s="6" t="n">
         <f aca="false">I6-J6</f>
-        <v>226.223245573025</v>
+        <v>122.285860253974</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1218,7 +1233,7 @@
       </c>
       <c r="C7" s="9" t="n">
         <f aca="false">SUM(C5:C6)</f>
-        <v>2394</v>
+        <v>2604</v>
       </c>
       <c r="D7" s="9" t="n">
         <f aca="false">SUM(D5:D6)</f>
@@ -1226,15 +1241,15 @@
       </c>
       <c r="E7" s="9" t="n">
         <f aca="false">SUM(E5:E6)</f>
-        <v>2422</v>
+        <v>2632</v>
       </c>
       <c r="F7" s="10" t="n">
         <f aca="false">IF(B7=0,0,E7/B7)</f>
-        <v>0.563255813953488</v>
+        <v>0.612093023255814</v>
       </c>
       <c r="G7" s="9" t="n">
         <f aca="false">SUM(G5:G6)</f>
-        <v>1878</v>
+        <v>1668</v>
       </c>
       <c r="H7" s="9" t="n">
         <f aca="false">SUM(H5:H6)</f>
@@ -1242,15 +1257,15 @@
       </c>
       <c r="I7" s="9" t="n">
         <f aca="false">SUM(I5:I6)</f>
-        <v>1442</v>
+        <v>1232</v>
       </c>
       <c r="J7" s="9" t="n">
         <f aca="false">SUM(J5:J6)</f>
-        <v>504.733026328093</v>
+        <v>472.914241923808</v>
       </c>
       <c r="K7" s="9" t="n">
         <f aca="false">SUM(K5:K6)</f>
-        <v>937.266973671907</v>
+        <v>759.085758076192</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1332,11 +1347,11 @@
       </c>
       <c r="I13" s="6" t="n">
         <f aca="false">IF($A13="","",IF($A13=Paramètres!$B$6,SUM($E$13:$E$22),IF($A13=Paramètres!$B$7,SUM($F$13:$F$22),0)))</f>
-        <v>1298.22324557302</v>
+        <v>1404.28586025397</v>
       </c>
       <c r="J13" s="6" t="n">
         <f aca="false">IF($A13="","",G13+D13+H13+IF(B13="Joint",E13+F13,0)-C13-I13)</f>
-        <v>1101.77675442698</v>
+        <v>995.714139746026</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1374,11 +1389,11 @@
       </c>
       <c r="I14" s="6" t="n">
         <f aca="false">IF($A14="","",IF($A14=Paramètres!$B$6,SUM($E$13:$E$22),IF($A14=Paramètres!$B$7,SUM($F$13:$F$22),0)))</f>
-        <v>1095.77675442698</v>
+        <v>1199.71413974603</v>
       </c>
       <c r="J14" s="6" t="n">
         <f aca="false">IF($A14="","",G14+D14+H14+IF(B14="Joint",E14+F14,0)-C14-I14)</f>
-        <v>776.223245573025</v>
+        <v>672.285860253974</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1434,7 +1449,7 @@
       </c>
       <c r="C16" s="6" t="n">
         <f aca="false">IF($A16="","",SUMIFS(Charges!$F$5:$F$54,Charges!$H$5:$H$54,$A16))</f>
-        <v>1160.66666666667</v>
+        <v>1370.66666666667</v>
       </c>
       <c r="D16" s="6" t="n">
         <f aca="false">IF($A16="","",SUMIFS(Revenus!$F$5:$F$24,Revenus!$G$5:$G$24,$A16,Revenus!$B$5:$B$24,"&lt;&gt;Salaire"))</f>
@@ -1442,11 +1457,11 @@
       </c>
       <c r="E16" s="11" t="n">
         <f aca="false">IF($A16="","",IF($B16="Joint",IF($C16=0,0,($C16-$D16)*SUMIFS(Charges!$M$5:$M$54,Charges!$H$5:$H$54,$A16)/$C16),0))</f>
-        <v>493.397664177676</v>
+        <v>599.460278858625</v>
       </c>
       <c r="F16" s="11" t="n">
         <f aca="false">IF($A16="","",IF($B16="Joint",IF($C16=0,0,($C16-$D16)*SUMIFS(Charges!$N$5:$N$54,Charges!$H$5:$H$54,$A16)/$C16),0))</f>
-        <v>437.269002488991</v>
+        <v>541.206387808042</v>
       </c>
       <c r="G16" s="6" t="n">
         <f aca="false">IF($A16="","",SUMIFS(Revenus!$F$5:$F$24,Revenus!$G$5:$G$24,$A16,Revenus!$B$5:$B$24,"Salaire"))</f>
@@ -1724,7 +1739,7 @@
       <c r="B23" s="8"/>
       <c r="C23" s="9" t="n">
         <f aca="false">SUM(C13:C22)</f>
-        <v>2652</v>
+        <v>2862</v>
       </c>
       <c r="D23" s="9" t="n">
         <f aca="false">SUM(D13:D22)</f>
@@ -1732,11 +1747,11 @@
       </c>
       <c r="E23" s="9" t="n">
         <f aca="false">SUM(E13:E22)</f>
-        <v>1298.22324557302</v>
+        <v>1404.28586025397</v>
       </c>
       <c r="F23" s="9" t="n">
         <f aca="false">SUM(F13:F22)</f>
-        <v>1095.77675442698</v>
+        <v>1199.71413974603</v>
       </c>
       <c r="G23" s="9" t="n">
         <f aca="false">SUM(G13:G22)</f>
@@ -1748,11 +1763,11 @@
       </c>
       <c r="I23" s="9" t="n">
         <f aca="false">SUM(I13:I22)</f>
-        <v>2394</v>
+        <v>2604</v>
       </c>
       <c r="J23" s="9" t="n">
         <f aca="false">SUM(J13:J22)</f>
-        <v>2157</v>
+        <v>1947</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1771,11 +1786,11 @@
       </c>
       <c r="B28" s="6" t="n">
         <f aca="false">SUMIFS(Charges!$F$5:$F$54,Charges!$C$5:$C$54,"Fixe")</f>
-        <v>1581.33333333333</v>
+        <v>1731.33333333333</v>
       </c>
       <c r="C28" s="7" t="n">
         <f aca="false">IF($B$30=0,0,B28/$B$30)</f>
-        <v>0.596279537456008</v>
+        <v>0.604938271604938</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1784,11 +1799,11 @@
       </c>
       <c r="B29" s="6" t="n">
         <f aca="false">SUMIFS(Charges!$F$5:$F$54,Charges!$C$5:$C$54,"Variable")</f>
-        <v>1070.66666666667</v>
+        <v>1130.66666666667</v>
       </c>
       <c r="C29" s="7" t="n">
         <f aca="false">IF($B$30=0,0,B29/$B$30)</f>
-        <v>0.403720462543992</v>
+        <v>0.395061728395062</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1797,7 +1812,7 @@
       </c>
       <c r="B30" s="9" t="n">
         <f aca="false">B28+B29</f>
-        <v>2652</v>
+        <v>2862</v>
       </c>
       <c r="C30" s="10" t="n">
         <f aca="false">C28+C29</f>
@@ -2922,87 +2937,139 @@
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="13"/>
-      <c r="B19" s="13"/>
-      <c r="C19" s="13"/>
-      <c r="D19" s="13"/>
-      <c r="E19" s="18"/>
-      <c r="F19" s="6" t="str">
+      <c r="A19" s="13" t="s">
+        <v>129</v>
+      </c>
+      <c r="B19" s="13" t="s">
+        <v>130</v>
+      </c>
+      <c r="C19" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="D19" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="E19" s="18" t="n">
+        <v>120</v>
+      </c>
+      <c r="F19" s="6" t="n">
         <f aca="false">IF(A19="","",IFERROR(E19/INDEX(Paramètres!$E$4:$E$7,MATCH(D19,Paramètres!$D$4:$D$7,0)),0))</f>
-        <v/>
-      </c>
-      <c r="G19" s="13"/>
-      <c r="H19" s="13"/>
+        <v>120</v>
+      </c>
+      <c r="G19" s="13" t="s">
+        <v>131</v>
+      </c>
+      <c r="H19" s="13" t="s">
+        <v>74</v>
+      </c>
       <c r="I19" s="13"/>
-      <c r="J19" s="13"/>
-      <c r="K19" s="13"/>
-      <c r="L19" s="7" t="str">
+      <c r="J19" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K19" s="13" t="s">
+        <v>101</v>
+      </c>
+      <c r="L19" s="7" t="n">
         <f aca="false">IF(A19="","",IF(K19="50/50",0.5,IF(K19="Prorata salaires",Paramètres!$B$9,IF(K19="Personne 1 seul",1,IF(K19="Personne 2 seul",0,0.5)))))</f>
-        <v/>
-      </c>
-      <c r="M19" s="6" t="str">
+        <v>0.5</v>
+      </c>
+      <c r="M19" s="6" t="n">
         <f aca="false">IF(A19="","",F19*L19)</f>
-        <v/>
-      </c>
-      <c r="N19" s="6" t="str">
+        <v>60</v>
+      </c>
+      <c r="N19" s="6" t="n">
         <f aca="false">IF(A19="","",F19-M19)</f>
-        <v/>
+        <v>60</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="13"/>
-      <c r="B20" s="13"/>
-      <c r="C20" s="13"/>
-      <c r="D20" s="13"/>
-      <c r="E20" s="18"/>
-      <c r="F20" s="6" t="str">
+      <c r="A20" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="C20" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="D20" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="E20" s="18" t="n">
+        <v>30</v>
+      </c>
+      <c r="F20" s="6" t="n">
         <f aca="false">IF(A20="","",IFERROR(E20/INDEX(Paramètres!$E$4:$E$7,MATCH(D20,Paramètres!$D$4:$D$7,0)),0))</f>
-        <v/>
-      </c>
-      <c r="G20" s="13"/>
-      <c r="H20" s="13"/>
+        <v>30</v>
+      </c>
+      <c r="G20" s="13" t="s">
+        <v>131</v>
+      </c>
+      <c r="H20" s="13" t="s">
+        <v>74</v>
+      </c>
       <c r="I20" s="13"/>
-      <c r="J20" s="13"/>
-      <c r="K20" s="13"/>
-      <c r="L20" s="7" t="str">
+      <c r="J20" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K20" s="13" t="s">
+        <v>101</v>
+      </c>
+      <c r="L20" s="7" t="n">
         <f aca="false">IF(A20="","",IF(K20="50/50",0.5,IF(K20="Prorata salaires",Paramètres!$B$9,IF(K20="Personne 1 seul",1,IF(K20="Personne 2 seul",0,0.5)))))</f>
-        <v/>
-      </c>
-      <c r="M20" s="6" t="str">
+        <v>0.5</v>
+      </c>
+      <c r="M20" s="6" t="n">
         <f aca="false">IF(A20="","",F20*L20)</f>
-        <v/>
-      </c>
-      <c r="N20" s="6" t="str">
+        <v>15</v>
+      </c>
+      <c r="N20" s="6" t="n">
         <f aca="false">IF(A20="","",F20-M20)</f>
-        <v/>
+        <v>15</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="13"/>
-      <c r="B21" s="13"/>
-      <c r="C21" s="13"/>
-      <c r="D21" s="13"/>
-      <c r="E21" s="18"/>
-      <c r="F21" s="6" t="str">
+      <c r="A21" s="13" t="s">
+        <v>133</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>114</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>105</v>
+      </c>
+      <c r="D21" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="E21" s="18" t="n">
+        <v>60</v>
+      </c>
+      <c r="F21" s="6" t="n">
         <f aca="false">IF(A21="","",IFERROR(E21/INDEX(Paramètres!$E$4:$E$7,MATCH(D21,Paramètres!$D$4:$D$7,0)),0))</f>
-        <v/>
-      </c>
-      <c r="G21" s="13"/>
-      <c r="H21" s="13"/>
+        <v>60</v>
+      </c>
+      <c r="G21" s="13" t="s">
+        <v>131</v>
+      </c>
+      <c r="H21" s="13" t="s">
+        <v>74</v>
+      </c>
       <c r="I21" s="13"/>
       <c r="J21" s="13"/>
-      <c r="K21" s="13"/>
-      <c r="L21" s="7" t="str">
+      <c r="K21" s="13" t="s">
+        <v>101</v>
+      </c>
+      <c r="L21" s="7" t="n">
         <f aca="false">IF(A21="","",IF(K21="50/50",0.5,IF(K21="Prorata salaires",Paramètres!$B$9,IF(K21="Personne 1 seul",1,IF(K21="Personne 2 seul",0,0.5)))))</f>
-        <v/>
-      </c>
-      <c r="M21" s="6" t="str">
+        <v>0.5</v>
+      </c>
+      <c r="M21" s="6" t="n">
         <f aca="false">IF(A21="","",F21*L21)</f>
-        <v/>
-      </c>
-      <c r="N21" s="6" t="str">
+        <v>30</v>
+      </c>
+      <c r="N21" s="6" t="n">
         <f aca="false">IF(A21="","",F21-M21)</f>
-        <v/>
+        <v>30</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3931,19 +3998,19 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="22" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="F55" s="9" t="n">
         <f aca="false">SUM(F5:F54)</f>
-        <v>2652</v>
+        <v>2862</v>
       </c>
       <c r="M55" s="9" t="n">
         <f aca="false">SUM(M5:M54)</f>
-        <v>1420.15891472868</v>
+        <v>1525.15891472868</v>
       </c>
       <c r="N55" s="9" t="n">
         <f aca="false">SUM(N5:N54)</f>
-        <v>1231.84108527132</v>
+        <v>1336.84108527132</v>
       </c>
     </row>
   </sheetData>
@@ -3998,12 +4065,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4026,7 +4093,7 @@
         <v>89</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="H4" s="4" t="s">
         <v>93</v>
@@ -4034,10 +4101,10 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="C5" s="13" t="s">
         <v>35</v>
@@ -4061,10 +4128,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="C6" s="13" t="s">
         <v>38</v>
@@ -4088,13 +4155,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="D7" s="18" t="n">
         <v>140</v>
@@ -4115,13 +4182,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="D8" s="18" t="n">
         <v>270</v>
@@ -4350,7 +4417,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="22" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="F25" s="9" t="n">
         <f aca="false">SUM(F5:F24)</f>
@@ -4398,12 +4465,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4428,7 +4495,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="B5" s="13" t="s">
         <v>35</v>
@@ -4449,13 +4516,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="B6" s="13" t="s">
         <v>35</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="D6" s="13" t="s">
         <v>39</v>
@@ -4470,7 +4537,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="B7" s="13" t="s">
         <v>35</v>
@@ -4898,7 +4965,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="22" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="F45" s="9" t="n">
         <f aca="false">SUM(F5:F44)</f>
@@ -4907,12 +4974,12 @@
     </row>
   </sheetData>
   <dataValidations count="2">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B5:B44" type="list">
+      <formula1>Paramètres!$B$4:$B$5</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D5:D44" type="list">
       <formula1>"Mensuelle,Trimestrielle,Semestrielle,Annuelle"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B5:B44" type="list">
-      <formula1>Paramètres!$B$4:$B$5</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -4942,17 +5009,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="23" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="B4" s="6" t="n">
         <f aca="false">SUMIFS(Charges!$F$5:$F$54,Charges!$B$5:$B$54,"Imprévus")</f>
@@ -4961,7 +5028,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="23" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="B5" s="24" t="n">
         <v>46266</v>
@@ -4969,7 +5036,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="23" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="B6" s="18" t="n">
         <v>0</v>
@@ -4977,7 +5044,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="23" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="B7" s="25" t="n">
         <f aca="true">MAX(0,(YEAR(TODAY())-YEAR(B5))*12+MONTH(TODAY())-MONTH(B5)+1)</f>
@@ -4986,7 +5053,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="23" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="B8" s="6" t="n">
         <f aca="false">B6+B4*B7</f>
@@ -4995,7 +5062,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="23" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="B9" s="6" t="n">
         <f aca="false">SUM(C13:C62)</f>
@@ -5004,7 +5071,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="B10" s="9" t="n">
         <f aca="false">B8-B9</f>
@@ -5013,21 +5080,21 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>85</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5035,7 +5102,7 @@
         <v>46285</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="C13" s="18" t="n">
         <v>220</v>
@@ -5049,7 +5116,7 @@
         <v>46300</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="C14" s="18" t="n">
         <v>85</v>

</xml_diff>